<commit_message>
Separate UC (always-built, linked) from proposed (scenario toggle)
- New Supply forecast now = under-construction deliveries (linked from the
  Competitive Analysis roster, counted in every scenario) + proposed deliveries
  that are "built" under the selected demand scenario.
- Proposed pipeline gets a per-deal "Built In" dropdown (Bear/Base/Bull/None):
  a deal layers into the chosen scenario and all more-bearish (higher-supply)
  ones, so you can model "built only in the downside case". Default Bear.
- Pipeline blocks split into UNDER CONSTRUCTION (linked) and PROPOSED (toggle);
  reconciliation note compares scheduled UC vs CoStar's current UC units.
- Flag partial (QTD) as-of quarter: occupancy is point-in-time (valid), Y0 flow
  sums for that quarter are partial.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Bella_Mirage__Supply_Chart.xlsx
+++ b/output/Bella_Mirage__Supply_Chart.xlsx
@@ -298,9 +298,6 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -317,6 +314,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -9416,7 +9416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:W58"/>
+  <dimension ref="B2:X61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -9437,9 +9437,10 @@
     <col width="28" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="6" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
     <col width="8" customWidth="1" min="22" max="22"/>
     <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="6" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="2" ht="22" customHeight="1">
@@ -9452,7 +9453,7 @@
     <row r="3">
       <c r="R3" s="39" t="inlineStr">
         <is>
-          <t>PIPELINE INPUTS (forward new supply)</t>
+          <t>UNDER CONSTRUCTION (linked from Competitive Analysis)</t>
         </is>
       </c>
     </row>
@@ -9487,15 +9488,10 @@
       </c>
       <c r="U4" s="42" t="inlineStr">
         <is>
-          <t>Incl?</t>
+          <t>DelivIdx</t>
         </is>
       </c>
       <c r="V4" s="42" t="inlineStr">
-        <is>
-          <t>DelivIdx</t>
-        </is>
-      </c>
-      <c r="W4" s="42" t="inlineStr">
         <is>
           <t>HoldYr</t>
         </is>
@@ -9516,26 +9512,24 @@
         <f>IFERROR(VALUE(RIGHT($C$5,4))*4+MATCH(LEFT($C$5,2),{"Q1","Q2","Q3","Q4"},0)-1,0)</f>
         <v/>
       </c>
-      <c r="R5" s="44" t="inlineStr">
-        <is>
-          <t>Sheely Center Future Phase</t>
-        </is>
-      </c>
-      <c r="S5" s="45" t="n">
-        <v>697</v>
-      </c>
-      <c r="T5" s="46" t="inlineStr"/>
-      <c r="U5" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V5" s="47">
+      <c r="R5" s="44">
+        <f>'Competitive Analysis'!C69</f>
+        <v/>
+      </c>
+      <c r="S5" s="45">
+        <f>'Competitive Analysis'!D69</f>
+        <v/>
+      </c>
+      <c r="T5" s="46">
+        <f>'Competitive Analysis'!E69</f>
+        <v/>
+      </c>
+      <c r="U5" s="46">
         <f>IFERROR(VALUE(RIGHT(T5,4))*4+MATCH(LEFT(T5,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W5" s="47">
-        <f>IF(V5="","",IF(V5&lt;=$E$4,0,MAX(1,INT((V5-$E$5)/4)+1)))</f>
+      <c r="V5" s="46">
+        <f>IF(S5="","",IF(U5&lt;=$E$4,0,MAX(1,INT((U5-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9545,30 +9539,32 @@
           <t>Stabilization Target</t>
         </is>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="47">
         <f>Settings!$B$2</f>
         <v/>
       </c>
-      <c r="R6" s="44" t="inlineStr">
-        <is>
-          <t>Urban 95 Parcel C</t>
-        </is>
-      </c>
-      <c r="S6" s="45" t="n">
-        <v>500</v>
-      </c>
-      <c r="T6" s="46" t="inlineStr"/>
-      <c r="U6" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V6" s="47">
+      <c r="E6">
+        <f>IF($C$7="Bear",3,IF($C$7="Base",2,1))</f>
+        <v/>
+      </c>
+      <c r="R6" s="44">
+        <f>'Competitive Analysis'!C60</f>
+        <v/>
+      </c>
+      <c r="S6" s="45">
+        <f>'Competitive Analysis'!D60</f>
+        <v/>
+      </c>
+      <c r="T6" s="46">
+        <f>'Competitive Analysis'!E60</f>
+        <v/>
+      </c>
+      <c r="U6" s="46">
         <f>IFERROR(VALUE(RIGHT(T6,4))*4+MATCH(LEFT(T6,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W6" s="47">
-        <f>IF(V6="","",IF(V6&lt;=$E$4,0,MAX(1,INT((V6-$E$5)/4)+1)))</f>
+      <c r="V6" s="46">
+        <f>IF(S6="","",IF(U6&lt;=$E$4,0,MAX(1,INT((U6-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9583,26 +9579,24 @@
           <t>Base</t>
         </is>
       </c>
-      <c r="R7" s="44" t="inlineStr">
-        <is>
-          <t>Urban 95 Parcel B</t>
-        </is>
-      </c>
-      <c r="S7" s="45" t="n">
-        <v>478</v>
-      </c>
-      <c r="T7" s="46" t="inlineStr"/>
-      <c r="U7" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V7" s="47">
+      <c r="R7" s="44">
+        <f>'Competitive Analysis'!C64</f>
+        <v/>
+      </c>
+      <c r="S7" s="45">
+        <f>'Competitive Analysis'!D64</f>
+        <v/>
+      </c>
+      <c r="T7" s="46">
+        <f>'Competitive Analysis'!E64</f>
+        <v/>
+      </c>
+      <c r="U7" s="46">
         <f>IFERROR(VALUE(RIGHT(T7,4))*4+MATCH(LEFT(T7,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W7" s="47">
-        <f>IF(V7="","",IF(V7&lt;=$E$4,0,MAX(1,INT((V7-$E$5)/4)+1)))</f>
+      <c r="V7" s="46">
+        <f>IF(S7="","",IF(U7&lt;=$E$4,0,MAX(1,INT((U7-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9612,29 +9606,27 @@
           <t>Bear Annual Absorption</t>
         </is>
       </c>
-      <c r="C8" s="49" t="n">
+      <c r="C8" s="48" t="n">
         <v>1250</v>
       </c>
-      <c r="R8" s="44" t="inlineStr">
-        <is>
-          <t>Celebration Plaza Parcel B</t>
-        </is>
-      </c>
-      <c r="S8" s="45" t="n">
-        <v>410</v>
-      </c>
-      <c r="T8" s="46" t="inlineStr"/>
-      <c r="U8" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V8" s="47">
+      <c r="R8" s="44">
+        <f>'Competitive Analysis'!C62</f>
+        <v/>
+      </c>
+      <c r="S8" s="45">
+        <f>'Competitive Analysis'!D62</f>
+        <v/>
+      </c>
+      <c r="T8" s="46">
+        <f>'Competitive Analysis'!E62</f>
+        <v/>
+      </c>
+      <c r="U8" s="46">
         <f>IFERROR(VALUE(RIGHT(T8,4))*4+MATCH(LEFT(T8,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W8" s="47">
-        <f>IF(V8="","",IF(V8&lt;=$E$4,0,MAX(1,INT((V8-$E$5)/4)+1)))</f>
+      <c r="V8" s="46">
+        <f>IF(S8="","",IF(U8&lt;=$E$4,0,MAX(1,INT((U8-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9644,29 +9636,27 @@
           <t>Base Annual Absorption</t>
         </is>
       </c>
-      <c r="C9" s="49" t="n">
+      <c r="C9" s="48" t="n">
         <v>2525</v>
       </c>
-      <c r="R9" s="44" t="inlineStr">
-        <is>
-          <t>The District at Westgate</t>
-        </is>
-      </c>
-      <c r="S9" s="45" t="n">
-        <v>384</v>
-      </c>
-      <c r="T9" s="46" t="inlineStr"/>
-      <c r="U9" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V9" s="47">
+      <c r="R9" s="44">
+        <f>'Competitive Analysis'!C63</f>
+        <v/>
+      </c>
+      <c r="S9" s="45">
+        <f>'Competitive Analysis'!D63</f>
+        <v/>
+      </c>
+      <c r="T9" s="46">
+        <f>'Competitive Analysis'!E63</f>
+        <v/>
+      </c>
+      <c r="U9" s="46">
         <f>IFERROR(VALUE(RIGHT(T9,4))*4+MATCH(LEFT(T9,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W9" s="47">
-        <f>IF(V9="","",IF(V9&lt;=$E$4,0,MAX(1,INT((V9-$E$5)/4)+1)))</f>
+      <c r="V9" s="46">
+        <f>IF(S9="","",IF(U9&lt;=$E$4,0,MAX(1,INT((U9-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9676,29 +9666,27 @@
           <t>Bull Annual Absorption</t>
         </is>
       </c>
-      <c r="C10" s="49" t="n">
+      <c r="C10" s="48" t="n">
         <v>3800</v>
       </c>
-      <c r="R10" s="44" t="inlineStr">
-        <is>
-          <t>Picerne at Palm Valley</t>
-        </is>
-      </c>
-      <c r="S10" s="45" t="n">
-        <v>383</v>
-      </c>
-      <c r="T10" s="46" t="inlineStr"/>
-      <c r="U10" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V10" s="47">
+      <c r="R10" s="44">
+        <f>'Competitive Analysis'!C65</f>
+        <v/>
+      </c>
+      <c r="S10" s="45">
+        <f>'Competitive Analysis'!D65</f>
+        <v/>
+      </c>
+      <c r="T10" s="46">
+        <f>'Competitive Analysis'!E65</f>
+        <v/>
+      </c>
+      <c r="U10" s="46">
         <f>IFERROR(VALUE(RIGHT(T10,4))*4+MATCH(LEFT(T10,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W10" s="47">
-        <f>IF(V10="","",IF(V10&lt;=$E$4,0,MAX(1,INT((V10-$E$5)/4)+1)))</f>
+      <c r="V10" s="46">
+        <f>IF(S10="","",IF(U10&lt;=$E$4,0,MAX(1,INT((U10-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9708,30 +9696,28 @@
           <t>Selected Annual Demand</t>
         </is>
       </c>
-      <c r="C11" s="50">
+      <c r="C11" s="49">
         <f>IF($C$7="Bear",$C$8,IF($C$7="Bull",$C$10,$C$9))</f>
         <v/>
       </c>
-      <c r="R11" s="44" t="inlineStr">
-        <is>
-          <t>Liv Avondale</t>
-        </is>
-      </c>
-      <c r="S11" s="45" t="n">
-        <v>333</v>
-      </c>
-      <c r="T11" s="46" t="inlineStr"/>
-      <c r="U11" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V11" s="47">
+      <c r="R11" s="44">
+        <f>'Competitive Analysis'!C61</f>
+        <v/>
+      </c>
+      <c r="S11" s="45">
+        <f>'Competitive Analysis'!D61</f>
+        <v/>
+      </c>
+      <c r="T11" s="46">
+        <f>'Competitive Analysis'!E61</f>
+        <v/>
+      </c>
+      <c r="U11" s="46">
         <f>IFERROR(VALUE(RIGHT(T11,4))*4+MATCH(LEFT(T11,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W11" s="47">
-        <f>IF(V11="","",IF(V11&lt;=$E$4,0,MAX(1,INT((V11-$E$5)/4)+1)))</f>
+      <c r="V11" s="46">
+        <f>IF(S11="","",IF(U11&lt;=$E$4,0,MAX(1,INT((U11-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9741,29 +9727,27 @@
           <t>Occupied (as-of)</t>
         </is>
       </c>
-      <c r="C12" s="50" t="n">
+      <c r="C12" s="49" t="n">
         <v>22585</v>
       </c>
-      <c r="R12" s="44" t="inlineStr">
-        <is>
-          <t>Urban 95 Parcel A</t>
-        </is>
-      </c>
-      <c r="S12" s="45" t="n">
-        <v>324</v>
-      </c>
-      <c r="T12" s="46" t="inlineStr"/>
-      <c r="U12" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V12" s="47">
+      <c r="R12" s="44">
+        <f>'Competitive Analysis'!C68</f>
+        <v/>
+      </c>
+      <c r="S12" s="45">
+        <f>'Competitive Analysis'!D68</f>
+        <v/>
+      </c>
+      <c r="T12" s="46">
+        <f>'Competitive Analysis'!E68</f>
+        <v/>
+      </c>
+      <c r="U12" s="46">
         <f>IFERROR(VALUE(RIGHT(T12,4))*4+MATCH(LEFT(T12,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W12" s="47">
-        <f>IF(V12="","",IF(V12&lt;=$E$4,0,MAX(1,INT((V12-$E$5)/4)+1)))</f>
+      <c r="V12" s="46">
+        <f>IF(S12="","",IF(U12&lt;=$E$4,0,MAX(1,INT((U12-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
@@ -9773,106 +9757,57 @@
           <t>Inventory (as-of)</t>
         </is>
       </c>
-      <c r="C13" s="50" t="n">
+      <c r="C13" s="49" t="n">
         <v>26603</v>
       </c>
-      <c r="R13" s="44" t="inlineStr">
-        <is>
-          <t>The Waverly</t>
-        </is>
-      </c>
-      <c r="S13" s="45" t="n">
-        <v>323</v>
-      </c>
-      <c r="T13" s="46" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U13" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V13" s="47">
+      <c r="R13" s="44">
+        <f>'Competitive Analysis'!C66</f>
+        <v/>
+      </c>
+      <c r="S13" s="45">
+        <f>'Competitive Analysis'!D66</f>
+        <v/>
+      </c>
+      <c r="T13" s="46">
+        <f>'Competitive Analysis'!E66</f>
+        <v/>
+      </c>
+      <c r="U13" s="46">
         <f>IFERROR(VALUE(RIGHT(T13,4))*4+MATCH(LEFT(T13,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W13" s="47">
-        <f>IF(V13="","",IF(V13&lt;=$E$4,0,MAX(1,INT((V13-$E$5)/4)+1)))</f>
+      <c r="V13" s="46">
+        <f>IF(S13="","",IF(U13&lt;=$E$4,0,MAX(1,INT((U13-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="R14" s="44" t="inlineStr">
-        <is>
-          <t>Fuze 623</t>
-        </is>
-      </c>
-      <c r="S14" s="45" t="n">
-        <v>321</v>
-      </c>
-      <c r="T14" s="46" t="inlineStr"/>
-      <c r="U14" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V14" s="47">
+      <c r="R14" s="44">
+        <f>'Competitive Analysis'!C67</f>
+        <v/>
+      </c>
+      <c r="S14" s="45">
+        <f>'Competitive Analysis'!D67</f>
+        <v/>
+      </c>
+      <c r="T14" s="46">
+        <f>'Competitive Analysis'!E67</f>
+        <v/>
+      </c>
+      <c r="U14" s="46">
         <f>IFERROR(VALUE(RIGHT(T14,4))*4+MATCH(LEFT(T14,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W14" s="47">
-        <f>IF(V14="","",IF(V14&lt;=$E$4,0,MAX(1,INT((V14-$E$5)/4)+1)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="R15" s="44" t="inlineStr">
-        <is>
-          <t>Anton Glendale</t>
-        </is>
-      </c>
-      <c r="S15" s="45" t="n">
-        <v>320</v>
-      </c>
-      <c r="T15" s="46" t="inlineStr"/>
-      <c r="U15" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V15" s="47">
-        <f>IFERROR(VALUE(RIGHT(T15,4))*4+MATCH(LEFT(T15,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W15" s="47">
-        <f>IF(V15="","",IF(V15&lt;=$E$4,0,MAX(1,INT((V15-$E$5)/4)+1)))</f>
+      <c r="V14" s="46">
+        <f>IF(S14="","",IF(U14&lt;=$E$4,0,MAX(1,INT((U14-$E$5)/4)+1)))</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="R16" s="44" t="inlineStr">
-        <is>
-          <t>Western Garden II</t>
-        </is>
-      </c>
-      <c r="S16" s="45" t="n">
-        <v>314</v>
-      </c>
-      <c r="T16" s="46" t="inlineStr"/>
-      <c r="U16" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V16" s="47">
-        <f>IFERROR(VALUE(RIGHT(T16,4))*4+MATCH(LEFT(T16,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W16" s="47">
-        <f>IF(V16="","",IF(V16&lt;=$E$4,0,MAX(1,INT((V16-$E$5)/4)+1)))</f>
-        <v/>
+      <c r="R16" s="39" t="inlineStr">
+        <is>
+          <t>PROPOSED PIPELINE (scenario toggle)</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -9916,149 +9851,162 @@
           <t>Y0</t>
         </is>
       </c>
-      <c r="J17" s="51" t="inlineStr">
+      <c r="J17" s="50" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K17" s="51" t="inlineStr">
+      <c r="K17" s="50" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L17" s="51" t="inlineStr">
+      <c r="L17" s="50" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M17" s="51" t="inlineStr">
+      <c r="M17" s="50" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N17" s="51" t="inlineStr">
+      <c r="N17" s="50" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O17" s="51" t="inlineStr">
+      <c r="O17" s="50" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
-      <c r="R17" s="44" t="inlineStr">
-        <is>
-          <t>Sanctuair at Centerscape</t>
-        </is>
-      </c>
-      <c r="S17" s="45" t="n">
-        <v>303</v>
-      </c>
-      <c r="T17" s="46" t="inlineStr"/>
-      <c r="U17" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V17" s="47">
-        <f>IFERROR(VALUE(RIGHT(T17,4))*4+MATCH(LEFT(T17,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W17" s="47">
-        <f>IF(V17="","",IF(V17&lt;=$E$4,0,MAX(1,INT((V17-$E$5)/4)+1)))</f>
-        <v/>
+      <c r="R17" s="42" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="S17" s="42" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="T17" s="42" t="inlineStr">
+        <is>
+          <t>Est. Delivery</t>
+        </is>
+      </c>
+      <c r="U17" s="42" t="inlineStr">
+        <is>
+          <t>Built In</t>
+        </is>
+      </c>
+      <c r="V17" s="42" t="inlineStr">
+        <is>
+          <t>DelivIdx</t>
+        </is>
+      </c>
+      <c r="W17" s="42" t="inlineStr">
+        <is>
+          <t>HoldYr</t>
+        </is>
+      </c>
+      <c r="X17" s="42" t="inlineStr">
+        <is>
+          <t>Built?</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C18" s="51" t="inlineStr">
         <is>
           <t>Q3 2019–Q2 2020</t>
         </is>
       </c>
-      <c r="D18" s="52" t="inlineStr">
+      <c r="D18" s="51" t="inlineStr">
         <is>
           <t>Q3 2020–Q2 2021</t>
         </is>
       </c>
-      <c r="E18" s="52" t="inlineStr">
+      <c r="E18" s="51" t="inlineStr">
         <is>
           <t>Q3 2021–Q2 2022</t>
         </is>
       </c>
-      <c r="F18" s="52" t="inlineStr">
+      <c r="F18" s="51" t="inlineStr">
         <is>
           <t>Q3 2022–Q2 2023</t>
         </is>
       </c>
-      <c r="G18" s="52" t="inlineStr">
+      <c r="G18" s="51" t="inlineStr">
         <is>
           <t>Q3 2023–Q2 2024</t>
         </is>
       </c>
-      <c r="H18" s="52" t="inlineStr">
+      <c r="H18" s="51" t="inlineStr">
         <is>
           <t>Q3 2024–Q2 2025</t>
         </is>
       </c>
-      <c r="I18" s="52" t="inlineStr">
+      <c r="I18" s="51" t="inlineStr">
         <is>
           <t>Q3 2025–Q2 2026</t>
         </is>
       </c>
-      <c r="J18" s="52" t="inlineStr">
+      <c r="J18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 1</t>
         </is>
       </c>
-      <c r="K18" s="52" t="inlineStr">
+      <c r="K18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 2</t>
         </is>
       </c>
-      <c r="L18" s="52" t="inlineStr">
+      <c r="L18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 3</t>
         </is>
       </c>
-      <c r="M18" s="52" t="inlineStr">
+      <c r="M18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 4</t>
         </is>
       </c>
-      <c r="N18" s="52" t="inlineStr">
+      <c r="N18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 5</t>
         </is>
       </c>
-      <c r="O18" s="52" t="inlineStr">
+      <c r="O18" s="51" t="inlineStr">
         <is>
           <t>Hold Yr 6</t>
         </is>
       </c>
       <c r="R18" s="44" t="inlineStr">
         <is>
-          <t>Encore Avondale</t>
+          <t>Sheely Center Future Phase</t>
         </is>
       </c>
       <c r="S18" s="45" t="n">
-        <v>300</v>
-      </c>
-      <c r="T18" s="46" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U18" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V18" s="47">
+        <v>697</v>
+      </c>
+      <c r="T18" s="52" t="inlineStr"/>
+      <c r="U18" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V18" s="46">
         <f>IFERROR(VALUE(RIGHT(T18,4))*4+MATCH(LEFT(T18,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W18" s="47">
+      <c r="W18" s="46">
         <f>IF(V18="","",IF(V18&lt;=$E$4,0,MAX(1,INT((V18-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X18" s="46">
+        <f>IF(U18="None",0,IF($E$6&gt;=IF(U18="Bear",3,IF(U18="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10090,49 +10038,53 @@
         <v>1860</v>
       </c>
       <c r="J19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,1,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,1)+SUMIFS($S$18:$S$61,$W$18:$W$61,1,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="K19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,2,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,2)+SUMIFS($S$18:$S$61,$W$18:$W$61,2,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="L19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,3,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,3)+SUMIFS($S$18:$S$61,$W$18:$W$61,3,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="M19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,4,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,4)+SUMIFS($S$18:$S$61,$W$18:$W$61,4,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="N19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,5,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,5)+SUMIFS($S$18:$S$61,$W$18:$W$61,5,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="O19" s="54">
-        <f>SUMIFS($S$5:$S$58,$W$5:$W$58,6,$U$5:$U$58,"Y")</f>
+        <f>SUMIFS($S$5:$S$14,$V$5:$V$14,6)+SUMIFS($S$18:$S$61,$W$18:$W$61,6,$X$18:$X$61,1)</f>
         <v/>
       </c>
       <c r="R19" s="44" t="inlineStr">
         <is>
-          <t>Banyan Avondale</t>
+          <t>Urban 95 Parcel C</t>
         </is>
       </c>
       <c r="S19" s="45" t="n">
-        <v>296</v>
-      </c>
-      <c r="T19" s="46" t="inlineStr"/>
-      <c r="U19" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V19" s="47">
+        <v>500</v>
+      </c>
+      <c r="T19" s="52" t="inlineStr"/>
+      <c r="U19" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V19" s="46">
         <f>IFERROR(VALUE(RIGHT(T19,4))*4+MATCH(LEFT(T19,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W19" s="47">
+      <c r="W19" s="46">
         <f>IF(V19="","",IF(V19&lt;=$E$4,0,MAX(1,INT((V19-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X19" s="46">
+        <f>IF(U19="None",0,IF($E$6&gt;=IF(U19="Bear",3,IF(U19="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10189,24 +10141,28 @@
       </c>
       <c r="R20" s="44" t="inlineStr">
         <is>
-          <t>Rosilian Villas</t>
+          <t>Urban 95 Parcel B</t>
         </is>
       </c>
       <c r="S20" s="45" t="n">
-        <v>291</v>
-      </c>
-      <c r="T20" s="46" t="inlineStr"/>
-      <c r="U20" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V20" s="47">
+        <v>478</v>
+      </c>
+      <c r="T20" s="52" t="inlineStr"/>
+      <c r="U20" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V20" s="46">
         <f>IFERROR(VALUE(RIGHT(T20,4))*4+MATCH(LEFT(T20,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W20" s="47">
+      <c r="W20" s="46">
         <f>IF(V20="","",IF(V20&lt;=$E$4,0,MAX(1,INT((V20-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X20" s="46">
+        <f>IF(U20="None",0,IF($E$6&gt;=IF(U20="Bear",3,IF(U20="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10263,28 +10219,28 @@
       </c>
       <c r="R21" s="44" t="inlineStr">
         <is>
-          <t>The Statler at Estrella Parkway</t>
+          <t>Celebration Plaza Parcel B</t>
         </is>
       </c>
       <c r="S21" s="45" t="n">
-        <v>284</v>
-      </c>
-      <c r="T21" s="46" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U21" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V21" s="47">
+        <v>410</v>
+      </c>
+      <c r="T21" s="52" t="inlineStr"/>
+      <c r="U21" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V21" s="46">
         <f>IFERROR(VALUE(RIGHT(T21,4))*4+MATCH(LEFT(T21,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W21" s="47">
+      <c r="W21" s="46">
         <f>IF(V21="","",IF(V21&lt;=$E$4,0,MAX(1,INT((V21-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X21" s="46">
+        <f>IF(U21="None",0,IF($E$6&gt;=IF(U21="Bear",3,IF(U21="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10339,48 +10295,56 @@
       </c>
       <c r="R22" s="44" t="inlineStr">
         <is>
-          <t>Orion Avondale</t>
+          <t>The District at Westgate</t>
         </is>
       </c>
       <c r="S22" s="45" t="n">
-        <v>268</v>
-      </c>
-      <c r="T22" s="46" t="inlineStr"/>
-      <c r="U22" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V22" s="47">
+        <v>384</v>
+      </c>
+      <c r="T22" s="52" t="inlineStr"/>
+      <c r="U22" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V22" s="46">
         <f>IFERROR(VALUE(RIGHT(T22,4))*4+MATCH(LEFT(T22,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W22" s="47">
+      <c r="W22" s="46">
         <f>IF(V22="","",IF(V22&lt;=$E$4,0,MAX(1,INT((V22-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X22" s="46">
+        <f>IF(U22="None",0,IF($E$6&gt;=IF(U22="Bear",3,IF(U22="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="R23" s="44" t="inlineStr">
         <is>
-          <t>Tavalo at Avondale</t>
+          <t>Picerne at Palm Valley</t>
         </is>
       </c>
       <c r="S23" s="45" t="n">
-        <v>266</v>
-      </c>
-      <c r="T23" s="46" t="inlineStr"/>
-      <c r="U23" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V23" s="47">
+        <v>383</v>
+      </c>
+      <c r="T23" s="52" t="inlineStr"/>
+      <c r="U23" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V23" s="46">
         <f>IFERROR(VALUE(RIGHT(T23,4))*4+MATCH(LEFT(T23,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W23" s="47">
+      <c r="W23" s="46">
         <f>IF(V23="","",IF(V23&lt;=$E$4,0,MAX(1,INT((V23-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X23" s="46">
+        <f>IF(U23="None",0,IF($E$6&gt;=IF(U23="Bear",3,IF(U23="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10437,24 +10401,28 @@
       </c>
       <c r="R24" s="44" t="inlineStr">
         <is>
-          <t>Marbella Ranch East Future Phase</t>
+          <t>Liv Avondale</t>
         </is>
       </c>
       <c r="S24" s="45" t="n">
-        <v>266</v>
-      </c>
-      <c r="T24" s="46" t="inlineStr"/>
-      <c r="U24" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V24" s="47">
+        <v>333</v>
+      </c>
+      <c r="T24" s="52" t="inlineStr"/>
+      <c r="U24" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V24" s="46">
         <f>IFERROR(VALUE(RIGHT(T24,4))*4+MATCH(LEFT(T24,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W24" s="47">
+      <c r="W24" s="46">
         <f>IF(V24="","",IF(V24&lt;=$E$4,0,MAX(1,INT((V24-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X24" s="46">
+        <f>IF(U24="None",0,IF($E$6&gt;=IF(U24="Bear",3,IF(U24="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10511,48 +10479,60 @@
       </c>
       <c r="R25" s="44" t="inlineStr">
         <is>
-          <t>Crystal Cove</t>
+          <t>Urban 95 Parcel A</t>
         </is>
       </c>
       <c r="S25" s="45" t="n">
-        <v>260</v>
-      </c>
-      <c r="T25" s="46" t="inlineStr"/>
-      <c r="U25" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V25" s="47">
+        <v>324</v>
+      </c>
+      <c r="T25" s="52" t="inlineStr"/>
+      <c r="U25" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V25" s="46">
         <f>IFERROR(VALUE(RIGHT(T25,4))*4+MATCH(LEFT(T25,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W25" s="47">
+      <c r="W25" s="46">
         <f>IF(V25="","",IF(V25&lt;=$E$4,0,MAX(1,INT((V25-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X25" s="46">
+        <f>IF(U25="None",0,IF($E$6&gt;=IF(U25="Bear",3,IF(U25="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="R26" s="44" t="inlineStr">
         <is>
-          <t>Cornerstone at the Wigwam</t>
+          <t>The Waverly</t>
         </is>
       </c>
       <c r="S26" s="45" t="n">
-        <v>212</v>
-      </c>
-      <c r="T26" s="46" t="inlineStr"/>
-      <c r="U26" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V26" s="47">
+        <v>323</v>
+      </c>
+      <c r="T26" s="52" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U26" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V26" s="46">
         <f>IFERROR(VALUE(RIGHT(T26,4))*4+MATCH(LEFT(T26,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W26" s="47">
+      <c r="W26" s="46">
         <f>IF(V26="","",IF(V26&lt;=$E$4,0,MAX(1,INT((V26-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X26" s="46">
+        <f>IF(U26="None",0,IF($E$6&gt;=IF(U26="Bear",3,IF(U26="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10594,24 +10574,28 @@
       </c>
       <c r="R27" s="44" t="inlineStr">
         <is>
-          <t>Radia Avondale Station III</t>
+          <t>Fuze 623</t>
         </is>
       </c>
       <c r="S27" s="45" t="n">
-        <v>212</v>
-      </c>
-      <c r="T27" s="46" t="inlineStr"/>
-      <c r="U27" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V27" s="47">
+        <v>321</v>
+      </c>
+      <c r="T27" s="52" t="inlineStr"/>
+      <c r="U27" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V27" s="46">
         <f>IFERROR(VALUE(RIGHT(T27,4))*4+MATCH(LEFT(T27,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W27" s="47">
+      <c r="W27" s="46">
         <f>IF(V27="","",IF(V27&lt;=$E$4,0,MAX(1,INT((V27-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X27" s="46">
+        <f>IF(U27="None",0,IF($E$6&gt;=IF(U27="Bear",3,IF(U27="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10647,24 +10631,28 @@
       </c>
       <c r="R28" s="44" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel A</t>
+          <t>Anton Glendale</t>
         </is>
       </c>
       <c r="S28" s="45" t="n">
-        <v>181</v>
-      </c>
-      <c r="T28" s="46" t="inlineStr"/>
-      <c r="U28" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V28" s="47">
+        <v>320</v>
+      </c>
+      <c r="T28" s="52" t="inlineStr"/>
+      <c r="U28" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V28" s="46">
         <f>IFERROR(VALUE(RIGHT(T28,4))*4+MATCH(LEFT(T28,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W28" s="47">
+      <c r="W28" s="46">
         <f>IF(V28="","",IF(V28&lt;=$E$4,0,MAX(1,INT((V28-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X28" s="46">
+        <f>IF(U28="None",0,IF($E$6&gt;=IF(U28="Bear",3,IF(U28="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10700,24 +10688,28 @@
       </c>
       <c r="R29" s="44" t="inlineStr">
         <is>
-          <t>Villages at River Grove</t>
+          <t>Western Garden II</t>
         </is>
       </c>
       <c r="S29" s="45" t="n">
-        <v>180</v>
-      </c>
-      <c r="T29" s="46" t="inlineStr"/>
-      <c r="U29" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V29" s="47">
+        <v>314</v>
+      </c>
+      <c r="T29" s="52" t="inlineStr"/>
+      <c r="U29" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V29" s="46">
         <f>IFERROR(VALUE(RIGHT(T29,4))*4+MATCH(LEFT(T29,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W29" s="47">
+      <c r="W29" s="46">
         <f>IF(V29="","",IF(V29&lt;=$E$4,0,MAX(1,INT((V29-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X29" s="46">
+        <f>IF(U29="None",0,IF($E$6&gt;=IF(U29="Bear",3,IF(U29="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10753,48 +10745,60 @@
       </c>
       <c r="R30" s="44" t="inlineStr">
         <is>
-          <t>District 99</t>
+          <t>Sanctuair at Centerscape</t>
         </is>
       </c>
       <c r="S30" s="45" t="n">
-        <v>172</v>
-      </c>
-      <c r="T30" s="46" t="inlineStr"/>
-      <c r="U30" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V30" s="47">
+        <v>303</v>
+      </c>
+      <c r="T30" s="52" t="inlineStr"/>
+      <c r="U30" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V30" s="46">
         <f>IFERROR(VALUE(RIGHT(T30,4))*4+MATCH(LEFT(T30,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W30" s="47">
+      <c r="W30" s="46">
         <f>IF(V30="","",IF(V30&lt;=$E$4,0,MAX(1,INT((V30-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X30" s="46">
+        <f>IF(U30="None",0,IF($E$6&gt;=IF(U30="Bear",3,IF(U30="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="R31" s="44" t="inlineStr">
         <is>
-          <t>McDowell Villas</t>
+          <t>Encore Avondale</t>
         </is>
       </c>
       <c r="S31" s="45" t="n">
-        <v>164</v>
-      </c>
-      <c r="T31" s="46" t="inlineStr"/>
-      <c r="U31" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V31" s="47">
+        <v>300</v>
+      </c>
+      <c r="T31" s="52" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U31" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V31" s="46">
         <f>IFERROR(VALUE(RIGHT(T31,4))*4+MATCH(LEFT(T31,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W31" s="47">
+      <c r="W31" s="46">
         <f>IF(V31="","",IF(V31&lt;=$E$4,0,MAX(1,INT((V31-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X31" s="46">
+        <f>IF(U31="None",0,IF($E$6&gt;=IF(U31="Bear",3,IF(U31="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10836,24 +10840,28 @@
       </c>
       <c r="R32" s="44" t="inlineStr">
         <is>
-          <t>Avondale</t>
+          <t>Banyan Avondale</t>
         </is>
       </c>
       <c r="S32" s="45" t="n">
-        <v>156</v>
-      </c>
-      <c r="T32" s="46" t="inlineStr"/>
-      <c r="U32" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V32" s="47">
+        <v>296</v>
+      </c>
+      <c r="T32" s="52" t="inlineStr"/>
+      <c r="U32" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V32" s="46">
         <f>IFERROR(VALUE(RIGHT(T32,4))*4+MATCH(LEFT(T32,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W32" s="47">
+      <c r="W32" s="46">
         <f>IF(V32="","",IF(V32&lt;=$E$4,0,MAX(1,INT((V32-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X32" s="46">
+        <f>IF(U32="None",0,IF($E$6&gt;=IF(U32="Bear",3,IF(U32="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10883,24 +10891,28 @@
       </c>
       <c r="R33" s="44" t="inlineStr">
         <is>
-          <t>Porter Kyle Development</t>
+          <t>Rosilian Villas</t>
         </is>
       </c>
       <c r="S33" s="45" t="n">
-        <v>135</v>
-      </c>
-      <c r="T33" s="46" t="inlineStr"/>
-      <c r="U33" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V33" s="47">
+        <v>291</v>
+      </c>
+      <c r="T33" s="52" t="inlineStr"/>
+      <c r="U33" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V33" s="46">
         <f>IFERROR(VALUE(RIGHT(T33,4))*4+MATCH(LEFT(T33,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W33" s="47">
+      <c r="W33" s="46">
         <f>IF(V33="","",IF(V33&lt;=$E$4,0,MAX(1,INT((V33-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X33" s="46">
+        <f>IF(U33="None",0,IF($E$6&gt;=IF(U33="Bear",3,IF(U33="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10930,28 +10942,32 @@
       </c>
       <c r="R34" s="44" t="inlineStr">
         <is>
-          <t>Ascent Goodyear</t>
+          <t>The Statler at Estrella Parkway</t>
         </is>
       </c>
       <c r="S34" s="45" t="n">
-        <v>113</v>
-      </c>
-      <c r="T34" s="46" t="inlineStr">
+        <v>284</v>
+      </c>
+      <c r="T34" s="52" t="inlineStr">
         <is>
           <t>Q3 2028</t>
         </is>
       </c>
-      <c r="U34" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V34" s="47">
+      <c r="U34" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V34" s="46">
         <f>IFERROR(VALUE(RIGHT(T34,4))*4+MATCH(LEFT(T34,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W34" s="47">
+      <c r="W34" s="46">
         <f>IF(V34="","",IF(V34&lt;=$E$4,0,MAX(1,INT((V34-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X34" s="46">
+        <f>IF(U34="None",0,IF($E$6&gt;=IF(U34="Bear",3,IF(U34="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -10981,28 +10997,28 @@
       </c>
       <c r="R35" s="44" t="inlineStr">
         <is>
-          <t>Northern 107</t>
+          <t>Orion Avondale</t>
         </is>
       </c>
       <c r="S35" s="45" t="n">
-        <v>74</v>
-      </c>
-      <c r="T35" s="46" t="inlineStr">
-        <is>
-          <t>Q4 2028</t>
-        </is>
-      </c>
-      <c r="U35" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V35" s="47">
+        <v>268</v>
+      </c>
+      <c r="T35" s="52" t="inlineStr"/>
+      <c r="U35" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V35" s="46">
         <f>IFERROR(VALUE(RIGHT(T35,4))*4+MATCH(LEFT(T35,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W35" s="47">
+      <c r="W35" s="46">
         <f>IF(V35="","",IF(V35&lt;=$E$4,0,MAX(1,INT((V35-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X35" s="46">
+        <f>IF(U35="None",0,IF($E$6&gt;=IF(U35="Bear",3,IF(U35="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11014,24 +11030,28 @@
       </c>
       <c r="R36" s="44" t="inlineStr">
         <is>
-          <t>Zenn @ Sierra Verde</t>
+          <t>Tavalo at Avondale</t>
         </is>
       </c>
       <c r="S36" s="45" t="n">
-        <v>66</v>
-      </c>
-      <c r="T36" s="46" t="inlineStr"/>
-      <c r="U36" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V36" s="47">
+        <v>266</v>
+      </c>
+      <c r="T36" s="52" t="inlineStr"/>
+      <c r="U36" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V36" s="46">
         <f>IFERROR(VALUE(RIGHT(T36,4))*4+MATCH(LEFT(T36,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W36" s="47">
+      <c r="W36" s="46">
         <f>IF(V36="","",IF(V36&lt;=$E$4,0,MAX(1,INT((V36-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X36" s="46">
+        <f>IF(U36="None",0,IF($E$6&gt;=IF(U36="Bear",3,IF(U36="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11061,22 +11081,28 @@
       </c>
       <c r="R37" s="44" t="inlineStr">
         <is>
-          <t>The BLVD Residential District</t>
-        </is>
-      </c>
-      <c r="S37" s="45" t="n"/>
-      <c r="T37" s="46" t="inlineStr"/>
-      <c r="U37" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V37" s="47">
+          <t>Marbella Ranch East Future Phase</t>
+        </is>
+      </c>
+      <c r="S37" s="45" t="n">
+        <v>266</v>
+      </c>
+      <c r="T37" s="52" t="inlineStr"/>
+      <c r="U37" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V37" s="46">
         <f>IFERROR(VALUE(RIGHT(T37,4))*4+MATCH(LEFT(T37,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W37" s="47">
+      <c r="W37" s="46">
         <f>IF(V37="","",IF(V37&lt;=$E$4,0,MAX(1,INT((V37-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X37" s="46">
+        <f>IF(U37="None",0,IF($E$6&gt;=IF(U37="Bear",3,IF(U37="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11106,22 +11132,28 @@
       </c>
       <c r="R38" s="44" t="inlineStr">
         <is>
-          <t>The BLVD Park Avenue District</t>
-        </is>
-      </c>
-      <c r="S38" s="45" t="n"/>
-      <c r="T38" s="46" t="inlineStr"/>
-      <c r="U38" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V38" s="47">
+          <t>Crystal Cove</t>
+        </is>
+      </c>
+      <c r="S38" s="45" t="n">
+        <v>260</v>
+      </c>
+      <c r="T38" s="52" t="inlineStr"/>
+      <c r="U38" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V38" s="46">
         <f>IFERROR(VALUE(RIGHT(T38,4))*4+MATCH(LEFT(T38,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W38" s="47">
+      <c r="W38" s="46">
         <f>IF(V38="","",IF(V38&lt;=$E$4,0,MAX(1,INT((V38-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X38" s="46">
+        <f>IF(U38="None",0,IF($E$6&gt;=IF(U38="Bear",3,IF(U38="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11151,22 +11183,28 @@
       </c>
       <c r="R39" s="44" t="inlineStr">
         <is>
-          <t>Globe Land Investors Development</t>
-        </is>
-      </c>
-      <c r="S39" s="45" t="n"/>
-      <c r="T39" s="46" t="inlineStr"/>
-      <c r="U39" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V39" s="47">
+          <t>Cornerstone at the Wigwam</t>
+        </is>
+      </c>
+      <c r="S39" s="45" t="n">
+        <v>212</v>
+      </c>
+      <c r="T39" s="52" t="inlineStr"/>
+      <c r="U39" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V39" s="46">
         <f>IFERROR(VALUE(RIGHT(T39,4))*4+MATCH(LEFT(T39,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W39" s="47">
+      <c r="W39" s="46">
         <f>IF(V39="","",IF(V39&lt;=$E$4,0,MAX(1,INT((V39-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X39" s="46">
+        <f>IF(U39="None",0,IF($E$6&gt;=IF(U39="Bear",3,IF(U39="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11178,22 +11216,28 @@
       </c>
       <c r="R40" s="44" t="inlineStr">
         <is>
-          <t>Ball Park</t>
-        </is>
-      </c>
-      <c r="S40" s="45" t="n"/>
-      <c r="T40" s="46" t="inlineStr"/>
-      <c r="U40" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V40" s="47">
+          <t>Radia Avondale Station III</t>
+        </is>
+      </c>
+      <c r="S40" s="45" t="n">
+        <v>212</v>
+      </c>
+      <c r="T40" s="52" t="inlineStr"/>
+      <c r="U40" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V40" s="46">
         <f>IFERROR(VALUE(RIGHT(T40,4))*4+MATCH(LEFT(T40,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W40" s="47">
+      <c r="W40" s="46">
         <f>IF(V40="","",IF(V40&lt;=$E$4,0,MAX(1,INT((V40-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X40" s="46">
+        <f>IF(U40="None",0,IF($E$6&gt;=IF(U40="Bear",3,IF(U40="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11229,22 +11273,28 @@
       </c>
       <c r="R41" s="44" t="inlineStr">
         <is>
-          <t>Vision 2 Parcel A</t>
-        </is>
-      </c>
-      <c r="S41" s="45" t="n"/>
-      <c r="T41" s="46" t="inlineStr"/>
-      <c r="U41" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V41" s="47">
+          <t>Celebration Plaza Parcel A</t>
+        </is>
+      </c>
+      <c r="S41" s="45" t="n">
+        <v>181</v>
+      </c>
+      <c r="T41" s="52" t="inlineStr"/>
+      <c r="U41" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V41" s="46">
         <f>IFERROR(VALUE(RIGHT(T41,4))*4+MATCH(LEFT(T41,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W41" s="47">
+      <c r="W41" s="46">
         <f>IF(V41="","",IF(V41&lt;=$E$4,0,MAX(1,INT((V41-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X41" s="46">
+        <f>IF(U41="None",0,IF($E$6&gt;=IF(U41="Bear",3,IF(U41="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11280,22 +11330,28 @@
       </c>
       <c r="R42" s="44" t="inlineStr">
         <is>
-          <t>Firststreet Verde</t>
-        </is>
-      </c>
-      <c r="S42" s="45" t="n"/>
-      <c r="T42" s="46" t="inlineStr"/>
-      <c r="U42" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V42" s="47">
+          <t>Villages at River Grove</t>
+        </is>
+      </c>
+      <c r="S42" s="45" t="n">
+        <v>180</v>
+      </c>
+      <c r="T42" s="52" t="inlineStr"/>
+      <c r="U42" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V42" s="46">
         <f>IFERROR(VALUE(RIGHT(T42,4))*4+MATCH(LEFT(T42,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W42" s="47">
+      <c r="W42" s="46">
         <f>IF(V42="","",IF(V42&lt;=$E$4,0,MAX(1,INT((V42-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X42" s="46">
+        <f>IF(U42="None",0,IF($E$6&gt;=IF(U42="Bear",3,IF(U42="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11331,422 +11387,531 @@
       </c>
       <c r="R43" s="44" t="inlineStr">
         <is>
-          <t>Goodyear Civic Square at Estrella Falls</t>
-        </is>
-      </c>
-      <c r="S43" s="45" t="n"/>
-      <c r="T43" s="46" t="inlineStr"/>
-      <c r="U43" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V43" s="47">
+          <t>District 99</t>
+        </is>
+      </c>
+      <c r="S43" s="45" t="n">
+        <v>172</v>
+      </c>
+      <c r="T43" s="52" t="inlineStr"/>
+      <c r="U43" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V43" s="46">
         <f>IFERROR(VALUE(RIGHT(T43,4))*4+MATCH(LEFT(T43,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W43" s="47">
+      <c r="W43" s="46">
         <f>IF(V43="","",IF(V43&lt;=$E$4,0,MAX(1,INT((V43-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X43" s="46">
+        <f>IF(U43="None",0,IF($E$6&gt;=IF(U43="Bear",3,IF(U43="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="33" t="inlineStr">
         <is>
-          <t>Reconciliation: scheduled pipeline (Incl=Y) vs CoStar Under Construction = 1,251 units.</t>
+          <t>Reconciliation: UC pipeline scheduled = 1,947 units vs CoStar current Under Construction = 1,251 units.</t>
         </is>
       </c>
       <c r="R44" s="44" t="inlineStr">
         <is>
-          <t>I-10 Innovation Center II</t>
-        </is>
-      </c>
-      <c r="S44" s="45" t="n"/>
-      <c r="T44" s="46" t="inlineStr"/>
-      <c r="U44" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V44" s="47">
+          <t>McDowell Villas</t>
+        </is>
+      </c>
+      <c r="S44" s="45" t="n">
+        <v>164</v>
+      </c>
+      <c r="T44" s="52" t="inlineStr"/>
+      <c r="U44" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V44" s="46">
         <f>IFERROR(VALUE(RIGHT(T44,4))*4+MATCH(LEFT(T44,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W44" s="47">
+      <c r="W44" s="46">
         <f>IF(V44="","",IF(V44&lt;=$E$4,0,MAX(1,INT((V44-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X44" s="46">
+        <f>IF(U44="None",0,IF($E$6&gt;=IF(U44="Bear",3,IF(U44="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="33" t="inlineStr">
         <is>
-          <t>Historical = CoStar 5-mi TTM actuals. Forecast: inventory += scheduled pipeline; occupied += selected demand (capped at target). Edit yellow cells (close quarter, demand scenario/levels, pipeline dates &amp; include, rent-growth &amp; concessions).</t>
+          <t>Note: as-of quarter (2026 Q2 QTD) is partial (quarter-to-date). Occupancy is point-in-time (valid); Y0 supply/absorption sums for that quarter are partial.</t>
         </is>
       </c>
       <c r="R45" s="44" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel D</t>
-        </is>
-      </c>
-      <c r="S45" s="45" t="n"/>
-      <c r="T45" s="46" t="inlineStr"/>
-      <c r="U45" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V45" s="47">
+          <t>Avondale</t>
+        </is>
+      </c>
+      <c r="S45" s="45" t="n">
+        <v>156</v>
+      </c>
+      <c r="T45" s="52" t="inlineStr"/>
+      <c r="U45" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V45" s="46">
         <f>IFERROR(VALUE(RIGHT(T45,4))*4+MATCH(LEFT(T45,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W45" s="47">
+      <c r="W45" s="46">
         <f>IF(V45="","",IF(V45&lt;=$E$4,0,MAX(1,INT((V45-$E$5)/4)+1)))</f>
         <v/>
       </c>
+      <c r="X45" s="46">
+        <f>IF(U45="None",0,IF($E$6&gt;=IF(U45="Bear",3,IF(U45="Base",2,1)),1,0))</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
+      <c r="B46" s="33" t="inlineStr">
+        <is>
+          <t>Historical = CoStar 5-mi TTM actuals. Forecast: inventory += UC (linked from Competitive Analysis) + proposed built this scenario; occupied += selected demand (capped at target). Yellow cells are editable.</t>
+        </is>
+      </c>
       <c r="R46" s="44" t="inlineStr">
         <is>
-          <t>SimonMed Development II</t>
-        </is>
-      </c>
-      <c r="S46" s="45" t="n"/>
-      <c r="T46" s="46" t="inlineStr"/>
-      <c r="U46" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V46" s="47">
+          <t>Porter Kyle Development</t>
+        </is>
+      </c>
+      <c r="S46" s="45" t="n">
+        <v>135</v>
+      </c>
+      <c r="T46" s="52" t="inlineStr"/>
+      <c r="U46" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V46" s="46">
         <f>IFERROR(VALUE(RIGHT(T46,4))*4+MATCH(LEFT(T46,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W46" s="47">
+      <c r="W46" s="46">
         <f>IF(V46="","",IF(V46&lt;=$E$4,0,MAX(1,INT((V46-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X46" s="46">
+        <f>IF(U46="None",0,IF($E$6&gt;=IF(U46="Bear",3,IF(U46="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="R47" s="44" t="inlineStr">
         <is>
-          <t>182 South 95th Avenue</t>
-        </is>
-      </c>
-      <c r="S47" s="45" t="n"/>
-      <c r="T47" s="46" t="inlineStr"/>
-      <c r="U47" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V47" s="47">
+          <t>Ascent Goodyear</t>
+        </is>
+      </c>
+      <c r="S47" s="45" t="n">
+        <v>113</v>
+      </c>
+      <c r="T47" s="52" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U47" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V47" s="46">
         <f>IFERROR(VALUE(RIGHT(T47,4))*4+MATCH(LEFT(T47,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W47" s="47">
+      <c r="W47" s="46">
         <f>IF(V47="","",IF(V47&lt;=$E$4,0,MAX(1,INT((V47-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X47" s="46">
+        <f>IF(U47="None",0,IF($E$6&gt;=IF(U47="Bear",3,IF(U47="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="R48" s="44" t="inlineStr">
         <is>
-          <t>Envision Encore</t>
-        </is>
-      </c>
-      <c r="S48" s="45" t="n"/>
-      <c r="T48" s="46" t="inlineStr"/>
-      <c r="U48" s="46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="V48" s="47">
+          <t>Northern 107</t>
+        </is>
+      </c>
+      <c r="S48" s="45" t="n">
+        <v>74</v>
+      </c>
+      <c r="T48" s="52" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="U48" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V48" s="46">
         <f>IFERROR(VALUE(RIGHT(T48,4))*4+MATCH(LEFT(T48,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W48" s="47">
+      <c r="W48" s="46">
         <f>IF(V48="","",IF(V48&lt;=$E$4,0,MAX(1,INT((V48-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X48" s="46">
+        <f>IF(U48="None",0,IF($E$6&gt;=IF(U48="Bear",3,IF(U48="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="R49" s="44" t="inlineStr">
         <is>
-          <t>FUZE Ballpark</t>
+          <t>Zenn @ Sierra Verde</t>
         </is>
       </c>
       <c r="S49" s="45" t="n">
-        <v>321</v>
-      </c>
-      <c r="T49" s="46" t="inlineStr">
-        <is>
-          <t>Q3 2026</t>
-        </is>
-      </c>
-      <c r="U49" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V49" s="47">
+        <v>66</v>
+      </c>
+      <c r="T49" s="52" t="inlineStr"/>
+      <c r="U49" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V49" s="46">
         <f>IFERROR(VALUE(RIGHT(T49,4))*4+MATCH(LEFT(T49,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W49" s="47">
+      <c r="W49" s="46">
         <f>IF(V49="","",IF(V49&lt;=$E$4,0,MAX(1,INT((V49-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X49" s="46">
+        <f>IF(U49="None",0,IF($E$6&gt;=IF(U49="Bear",3,IF(U49="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="R50" s="44" t="inlineStr">
         <is>
-          <t>Zanjero III</t>
-        </is>
-      </c>
-      <c r="S50" s="45" t="n">
-        <v>301</v>
-      </c>
-      <c r="T50" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2028</t>
-        </is>
-      </c>
-      <c r="U50" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V50" s="47">
+          <t>The BLVD Residential District</t>
+        </is>
+      </c>
+      <c r="S50" s="45" t="n"/>
+      <c r="T50" s="52" t="inlineStr"/>
+      <c r="U50" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V50" s="46">
         <f>IFERROR(VALUE(RIGHT(T50,4))*4+MATCH(LEFT(T50,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W50" s="47">
+      <c r="W50" s="46">
         <f>IF(V50="","",IF(V50&lt;=$E$4,0,MAX(1,INT((V50-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X50" s="46">
+        <f>IF(U50="None",0,IF($E$6&gt;=IF(U50="Bear",3,IF(U50="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="R51" s="44" t="inlineStr">
         <is>
-          <t>Pointe Grand Estrella at Phoenix</t>
-        </is>
-      </c>
-      <c r="S51" s="45" t="n">
-        <v>288</v>
-      </c>
-      <c r="T51" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2027</t>
-        </is>
-      </c>
-      <c r="U51" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V51" s="47">
+          <t>The BLVD Park Avenue District</t>
+        </is>
+      </c>
+      <c r="S51" s="45" t="n"/>
+      <c r="T51" s="52" t="inlineStr"/>
+      <c r="U51" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V51" s="46">
         <f>IFERROR(VALUE(RIGHT(T51,4))*4+MATCH(LEFT(T51,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W51" s="47">
+      <c r="W51" s="46">
         <f>IF(V51="","",IF(V51&lt;=$E$4,0,MAX(1,INT((V51-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X51" s="46">
+        <f>IF(U51="None",0,IF($E$6&gt;=IF(U51="Bear",3,IF(U51="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="R52" s="44" t="inlineStr">
         <is>
-          <t>Yardly Algodon</t>
-        </is>
-      </c>
-      <c r="S52" s="45" t="n">
-        <v>262</v>
-      </c>
-      <c r="T52" s="46" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="U52" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V52" s="47">
+          <t>Globe Land Investors Development</t>
+        </is>
+      </c>
+      <c r="S52" s="45" t="n"/>
+      <c r="T52" s="52" t="inlineStr"/>
+      <c r="U52" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V52" s="46">
         <f>IFERROR(VALUE(RIGHT(T52,4))*4+MATCH(LEFT(T52,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W52" s="47">
+      <c r="W52" s="46">
         <f>IF(V52="","",IF(V52&lt;=$E$4,0,MAX(1,INT((V52-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X52" s="46">
+        <f>IF(U52="None",0,IF($E$6&gt;=IF(U52="Bear",3,IF(U52="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="R53" s="44" t="inlineStr">
         <is>
-          <t>Cerro Vista</t>
-        </is>
-      </c>
-      <c r="S53" s="45" t="n">
-        <v>255</v>
-      </c>
-      <c r="T53" s="46" t="inlineStr">
-        <is>
-          <t>Q4 2027</t>
-        </is>
-      </c>
-      <c r="U53" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V53" s="47">
+          <t>Ball Park</t>
+        </is>
+      </c>
+      <c r="S53" s="45" t="n"/>
+      <c r="T53" s="52" t="inlineStr"/>
+      <c r="U53" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V53" s="46">
         <f>IFERROR(VALUE(RIGHT(T53,4))*4+MATCH(LEFT(T53,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W53" s="47">
+      <c r="W53" s="46">
         <f>IF(V53="","",IF(V53&lt;=$E$4,0,MAX(1,INT((V53-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X53" s="46">
+        <f>IF(U53="None",0,IF($E$6&gt;=IF(U53="Bear",3,IF(U53="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="R54" s="44" t="inlineStr">
         <is>
-          <t>Marbella Ranch East I</t>
-        </is>
-      </c>
-      <c r="S54" s="45" t="n">
-        <v>144</v>
-      </c>
-      <c r="T54" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2027</t>
-        </is>
-      </c>
-      <c r="U54" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V54" s="47">
+          <t>Vision 2 Parcel A</t>
+        </is>
+      </c>
+      <c r="S54" s="45" t="n"/>
+      <c r="T54" s="52" t="inlineStr"/>
+      <c r="U54" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V54" s="46">
         <f>IFERROR(VALUE(RIGHT(T54,4))*4+MATCH(LEFT(T54,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W54" s="47">
+      <c r="W54" s="46">
         <f>IF(V54="","",IF(V54&lt;=$E$4,0,MAX(1,INT((V54-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X54" s="46">
+        <f>IF(U54="None",0,IF($E$6&gt;=IF(U54="Bear",3,IF(U54="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="R55" s="44" t="inlineStr">
         <is>
-          <t>Zen @ Angelina</t>
-        </is>
-      </c>
-      <c r="S55" s="45" t="n">
-        <v>130</v>
-      </c>
-      <c r="T55" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2028</t>
-        </is>
-      </c>
-      <c r="U55" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V55" s="47">
+          <t>Firststreet Verde</t>
+        </is>
+      </c>
+      <c r="S55" s="45" t="n"/>
+      <c r="T55" s="52" t="inlineStr"/>
+      <c r="U55" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V55" s="46">
         <f>IFERROR(VALUE(RIGHT(T55,4))*4+MATCH(LEFT(T55,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W55" s="47">
+      <c r="W55" s="46">
         <f>IF(V55="","",IF(V55&lt;=$E$4,0,MAX(1,INT((V55-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X55" s="46">
+        <f>IF(U55="None",0,IF($E$6&gt;=IF(U55="Bear",3,IF(U55="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="R56" s="44" t="inlineStr">
         <is>
-          <t>HARMON Ascend</t>
-        </is>
-      </c>
-      <c r="S56" s="45" t="n">
-        <v>125</v>
-      </c>
-      <c r="T56" s="46" t="inlineStr">
-        <is>
-          <t>Q1 2027</t>
-        </is>
-      </c>
-      <c r="U56" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V56" s="47">
+          <t>Goodyear Civic Square at Estrella Falls</t>
+        </is>
+      </c>
+      <c r="S56" s="45" t="n"/>
+      <c r="T56" s="52" t="inlineStr"/>
+      <c r="U56" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V56" s="46">
         <f>IFERROR(VALUE(RIGHT(T56,4))*4+MATCH(LEFT(T56,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W56" s="47">
+      <c r="W56" s="46">
         <f>IF(V56="","",IF(V56&lt;=$E$4,0,MAX(1,INT((V56-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X56" s="46">
+        <f>IF(U56="None",0,IF($E$6&gt;=IF(U56="Bear",3,IF(U56="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="R57" s="44" t="inlineStr">
         <is>
-          <t>Villages at Northern</t>
-        </is>
-      </c>
-      <c r="S57" s="45" t="n">
-        <v>74</v>
-      </c>
-      <c r="T57" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2027</t>
-        </is>
-      </c>
-      <c r="U57" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V57" s="47">
+          <t>I-10 Innovation Center II</t>
+        </is>
+      </c>
+      <c r="S57" s="45" t="n"/>
+      <c r="T57" s="52" t="inlineStr"/>
+      <c r="U57" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V57" s="46">
         <f>IFERROR(VALUE(RIGHT(T57,4))*4+MATCH(LEFT(T57,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W57" s="47">
+      <c r="W57" s="46">
         <f>IF(V57="","",IF(V57&lt;=$E$4,0,MAX(1,INT((V57-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X57" s="46">
+        <f>IF(U57="None",0,IF($E$6&gt;=IF(U57="Bear",3,IF(U57="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="R58" s="44" t="inlineStr">
         <is>
-          <t>Prosper 47</t>
-        </is>
-      </c>
-      <c r="S58" s="45" t="n">
-        <v>47</v>
-      </c>
-      <c r="T58" s="46" t="inlineStr">
-        <is>
-          <t>Q2 2027</t>
-        </is>
-      </c>
-      <c r="U58" s="46" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V58" s="47">
+          <t>Celebration Plaza Parcel D</t>
+        </is>
+      </c>
+      <c r="S58" s="45" t="n"/>
+      <c r="T58" s="52" t="inlineStr"/>
+      <c r="U58" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V58" s="46">
         <f>IFERROR(VALUE(RIGHT(T58,4))*4+MATCH(LEFT(T58,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
         <v/>
       </c>
-      <c r="W58" s="47">
+      <c r="W58" s="46">
         <f>IF(V58="","",IF(V58&lt;=$E$4,0,MAX(1,INT((V58-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X58" s="46">
+        <f>IF(U58="None",0,IF($E$6&gt;=IF(U58="Bear",3,IF(U58="Base",2,1)),1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="R59" s="44" t="inlineStr">
+        <is>
+          <t>SimonMed Development II</t>
+        </is>
+      </c>
+      <c r="S59" s="45" t="n"/>
+      <c r="T59" s="52" t="inlineStr"/>
+      <c r="U59" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V59" s="46">
+        <f>IFERROR(VALUE(RIGHT(T59,4))*4+MATCH(LEFT(T59,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W59" s="46">
+        <f>IF(V59="","",IF(V59&lt;=$E$4,0,MAX(1,INT((V59-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X59" s="46">
+        <f>IF(U59="None",0,IF($E$6&gt;=IF(U59="Bear",3,IF(U59="Base",2,1)),1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="R60" s="44" t="inlineStr">
+        <is>
+          <t>182 South 95th Avenue</t>
+        </is>
+      </c>
+      <c r="S60" s="45" t="n"/>
+      <c r="T60" s="52" t="inlineStr"/>
+      <c r="U60" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V60" s="46">
+        <f>IFERROR(VALUE(RIGHT(T60,4))*4+MATCH(LEFT(T60,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W60" s="46">
+        <f>IF(V60="","",IF(V60&lt;=$E$4,0,MAX(1,INT((V60-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X60" s="46">
+        <f>IF(U60="None",0,IF($E$6&gt;=IF(U60="Bear",3,IF(U60="Base",2,1)),1,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="R61" s="44" t="inlineStr">
+        <is>
+          <t>Envision Encore</t>
+        </is>
+      </c>
+      <c r="S61" s="45" t="n"/>
+      <c r="T61" s="52" t="inlineStr"/>
+      <c r="U61" s="52" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="V61" s="46">
+        <f>IFERROR(VALUE(RIGHT(T61,4))*4+MATCH(LEFT(T61,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W61" s="46">
+        <f>IF(V61="","",IF(V61&lt;=$E$4,0,MAX(1,INT((V61-$E$5)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X61" s="46">
+        <f>IF(U61="None",0,IF($E$6&gt;=IF(U61="Bear",3,IF(U61="Base",2,1)),1,0))</f>
         <v/>
       </c>
     </row>
@@ -11758,8 +11923,8 @@
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Bear,Base,Bull"</formula1>
     </dataValidation>
-    <dataValidation sqref="U5 U6 U7 U8 U9 U10 U11 U12 U13 U14 U15 U16 U17 U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Y,N"</formula1>
+    <dataValidation sqref="U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Bear,Base,Bull,None"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add subject rows (HelloData/CoStar rents + financials occupancy)
- New --intake input: parse the RR-T12 'Lease Trend' tab for subject market rent
  & effective rent (HelloData mix-weighted) and occupancy (T12 financials);
  aggregate to the relative-year TTM windows.
- New --costar-subject-rents input: CoStar per-property analytics used to extend
  subject rent history before HelloData coverage, level-aligned to HelloData via
  the overlap ratio (CoStar tracks the subject closer than RealPage).
- Add SUBJECT market rent / effective rent / occupancy rows under the 5-mi rows
  on the Supply & Absorption tab.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Bella_Mirage__Supply_Chart.xlsx
+++ b/output/Bella_Mirage__Supply_Chart.xlsx
@@ -19,9 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;;&quot;—&quot;"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -183,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -332,6 +333,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -10116,27 +10129,27 @@
         <v>2369</v>
       </c>
       <c r="J20" s="54">
-        <f>J25-I25</f>
+        <f>J29-I29</f>
         <v/>
       </c>
       <c r="K20" s="54">
-        <f>K25-J25</f>
+        <f>K29-J29</f>
         <v/>
       </c>
       <c r="L20" s="54">
-        <f>L25-K25</f>
+        <f>L29-K29</f>
         <v/>
       </c>
       <c r="M20" s="54">
-        <f>M25-L25</f>
+        <f>M29-L29</f>
         <v/>
       </c>
       <c r="N20" s="54">
-        <f>N25-M25</f>
+        <f>N29-M29</f>
         <v/>
       </c>
       <c r="O20" s="54">
-        <f>O25-N25</f>
+        <f>O29-N29</f>
         <v/>
       </c>
       <c r="R20" s="44" t="inlineStr">
@@ -10194,27 +10207,27 @@
         <v>0.849</v>
       </c>
       <c r="J21" s="56">
-        <f>IFERROR(J25/J24,0)</f>
+        <f>IFERROR(J29/J28,0)</f>
         <v/>
       </c>
       <c r="K21" s="56">
-        <f>IFERROR(K25/K24,0)</f>
+        <f>IFERROR(K29/K28,0)</f>
         <v/>
       </c>
       <c r="L21" s="56">
-        <f>IFERROR(L25/L24,0)</f>
+        <f>IFERROR(L29/L28,0)</f>
         <v/>
       </c>
       <c r="M21" s="56">
-        <f>IFERROR(M25/M24,0)</f>
+        <f>IFERROR(M29/M28,0)</f>
         <v/>
       </c>
       <c r="N21" s="56">
-        <f>IFERROR(N25/N24,0)</f>
+        <f>IFERROR(N29/N28,0)</f>
         <v/>
       </c>
       <c r="O21" s="56">
-        <f>IFERROR(O25/O24,0)</f>
+        <f>IFERROR(O29/O28,0)</f>
         <v/>
       </c>
       <c r="R21" s="44" t="inlineStr">
@@ -10321,6 +10334,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="B23" s="40" t="inlineStr">
+        <is>
+          <t>SUBJECT (Bella Mirage)</t>
+        </is>
+      </c>
       <c r="R23" s="44" t="inlineStr">
         <is>
           <t>Picerne at Palm Valley</t>
@@ -10348,57 +10366,39 @@
         <v/>
       </c>
     </row>
-    <row r="24" hidden="1">
-      <c r="B24" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  inventory</t>
-        </is>
-      </c>
-      <c r="C24" s="57" t="n">
-        <v>12401</v>
-      </c>
-      <c r="D24" s="57" t="n">
-        <v>14261</v>
-      </c>
-      <c r="E24" s="57" t="n">
-        <v>15597</v>
-      </c>
-      <c r="F24" s="57" t="n">
-        <v>17877</v>
-      </c>
-      <c r="G24" s="57" t="n">
-        <v>20700</v>
-      </c>
-      <c r="H24" s="57" t="n">
-        <v>24743</v>
-      </c>
-      <c r="I24" s="57" t="n">
-        <v>26603</v>
-      </c>
-      <c r="J24" s="57">
-        <f>I24+J19</f>
-        <v/>
-      </c>
-      <c r="K24" s="57">
-        <f>J24+K19</f>
-        <v/>
-      </c>
-      <c r="L24" s="57">
-        <f>K24+L19</f>
-        <v/>
-      </c>
-      <c r="M24" s="57">
-        <f>L24+M19</f>
-        <v/>
-      </c>
-      <c r="N24" s="57">
-        <f>M24+N19</f>
-        <v/>
-      </c>
-      <c r="O24" s="57">
-        <f>N24+O19</f>
-        <v/>
-      </c>
+    <row r="24">
+      <c r="B24" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Market Rent  (HD→CoStar)</t>
+        </is>
+      </c>
+      <c r="C24" s="58" t="n">
+        <v>1088</v>
+      </c>
+      <c r="D24" s="58" t="n">
+        <v>1437</v>
+      </c>
+      <c r="E24" s="58" t="n">
+        <v>1730</v>
+      </c>
+      <c r="F24" s="58" t="n">
+        <v>1572</v>
+      </c>
+      <c r="G24" s="58" t="n">
+        <v>1497</v>
+      </c>
+      <c r="H24" s="58" t="n">
+        <v>1444</v>
+      </c>
+      <c r="I24" s="58" t="n">
+        <v>1332</v>
+      </c>
+      <c r="J24" s="59" t="n"/>
+      <c r="K24" s="59" t="n"/>
+      <c r="L24" s="59" t="n"/>
+      <c r="M24" s="59" t="n"/>
+      <c r="N24" s="59" t="n"/>
+      <c r="O24" s="59" t="n"/>
       <c r="R24" s="44" t="inlineStr">
         <is>
           <t>Liv Avondale</t>
@@ -10426,57 +10426,39 @@
         <v/>
       </c>
     </row>
-    <row r="25" hidden="1">
-      <c r="B25" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  occupied</t>
-        </is>
-      </c>
-      <c r="C25" s="57" t="n">
-        <v>11277</v>
-      </c>
-      <c r="D25" s="57" t="n">
-        <v>13152</v>
-      </c>
-      <c r="E25" s="57" t="n">
-        <v>14362</v>
-      </c>
-      <c r="F25" s="57" t="n">
-        <v>15047</v>
-      </c>
-      <c r="G25" s="57" t="n">
-        <v>17560</v>
-      </c>
-      <c r="H25" s="57" t="n">
-        <v>20215</v>
-      </c>
-      <c r="I25" s="57" t="n">
-        <v>22585</v>
-      </c>
-      <c r="J25" s="57">
-        <f>MIN($C$6*J24,I25+$C$11)</f>
-        <v/>
-      </c>
-      <c r="K25" s="57">
-        <f>MIN($C$6*K24,J25+$C$11)</f>
-        <v/>
-      </c>
-      <c r="L25" s="57">
-        <f>MIN($C$6*L24,K25+$C$11)</f>
-        <v/>
-      </c>
-      <c r="M25" s="57">
-        <f>MIN($C$6*M24,L25+$C$11)</f>
-        <v/>
-      </c>
-      <c r="N25" s="57">
-        <f>MIN($C$6*N24,M25+$C$11)</f>
-        <v/>
-      </c>
-      <c r="O25" s="57">
-        <f>MIN($C$6*O24,N25+$C$11)</f>
-        <v/>
-      </c>
+    <row r="25">
+      <c r="B25" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Effective Rent</t>
+        </is>
+      </c>
+      <c r="C25" s="58" t="n">
+        <v>1086</v>
+      </c>
+      <c r="D25" s="58" t="n">
+        <v>1434</v>
+      </c>
+      <c r="E25" s="58" t="n">
+        <v>1730</v>
+      </c>
+      <c r="F25" s="58" t="n">
+        <v>1555</v>
+      </c>
+      <c r="G25" s="58" t="n">
+        <v>1402</v>
+      </c>
+      <c r="H25" s="58" t="n">
+        <v>1369</v>
+      </c>
+      <c r="I25" s="58" t="n">
+        <v>1301</v>
+      </c>
+      <c r="J25" s="59" t="n"/>
+      <c r="K25" s="59" t="n"/>
+      <c r="L25" s="59" t="n"/>
+      <c r="M25" s="59" t="n"/>
+      <c r="N25" s="59" t="n"/>
+      <c r="O25" s="59" t="n"/>
       <c r="R25" s="44" t="inlineStr">
         <is>
           <t>Urban 95 Parcel A</t>
@@ -10505,6 +10487,32 @@
       </c>
     </row>
     <row r="26">
+      <c r="B26" s="40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Occupancy (T12 financials)</t>
+        </is>
+      </c>
+      <c r="C26" s="60" t="n"/>
+      <c r="D26" s="60" t="n"/>
+      <c r="E26" s="60" t="n"/>
+      <c r="F26" s="60" t="n">
+        <v>0.8788971182681028</v>
+      </c>
+      <c r="G26" s="60" t="n">
+        <v>0.9173713229249606</v>
+      </c>
+      <c r="H26" s="60" t="n">
+        <v>0.9334854638634199</v>
+      </c>
+      <c r="I26" s="60" t="n">
+        <v>0.9206643232607364</v>
+      </c>
+      <c r="J26" s="61" t="n"/>
+      <c r="K26" s="61" t="n"/>
+      <c r="L26" s="61" t="n"/>
+      <c r="M26" s="61" t="n"/>
+      <c r="N26" s="61" t="n"/>
+      <c r="O26" s="61" t="n"/>
       <c r="R26" s="44" t="inlineStr">
         <is>
           <t>The Waverly</t>
@@ -10537,41 +10545,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="40" t="inlineStr">
-        <is>
-          <t>IMPLIED 5-MI OCCUPANCY BY DEMAND SCENARIO</t>
-        </is>
-      </c>
-      <c r="J27" s="58" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="K27" s="58" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="L27" s="58" t="inlineStr">
-        <is>
-          <t>Y3</t>
-        </is>
-      </c>
-      <c r="M27" s="58" t="inlineStr">
-        <is>
-          <t>Y4</t>
-        </is>
-      </c>
-      <c r="N27" s="58" t="inlineStr">
-        <is>
-          <t>Y5</t>
-        </is>
-      </c>
-      <c r="O27" s="58" t="inlineStr">
-        <is>
-          <t>Y6</t>
-        </is>
-      </c>
       <c r="R27" s="44" t="inlineStr">
         <is>
           <t>Fuze 623</t>
@@ -10599,34 +10572,55 @@
         <v/>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="40" t="inlineStr">
-        <is>
-          <t>Bear</t>
-        </is>
-      </c>
-      <c r="J28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*1)/J24)</f>
-        <v/>
-      </c>
-      <c r="K28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*2)/K24)</f>
-        <v/>
-      </c>
-      <c r="L28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*3)/L24)</f>
-        <v/>
-      </c>
-      <c r="M28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*4)/M24)</f>
-        <v/>
-      </c>
-      <c r="N28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*5)/N24)</f>
-        <v/>
-      </c>
-      <c r="O28" s="59">
-        <f>MIN($C$6,($C$12+$C$8*6)/O24)</f>
+    <row r="28" hidden="1">
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  inventory</t>
+        </is>
+      </c>
+      <c r="C28" s="57" t="n">
+        <v>12401</v>
+      </c>
+      <c r="D28" s="57" t="n">
+        <v>14261</v>
+      </c>
+      <c r="E28" s="57" t="n">
+        <v>15597</v>
+      </c>
+      <c r="F28" s="57" t="n">
+        <v>17877</v>
+      </c>
+      <c r="G28" s="57" t="n">
+        <v>20700</v>
+      </c>
+      <c r="H28" s="57" t="n">
+        <v>24743</v>
+      </c>
+      <c r="I28" s="57" t="n">
+        <v>26603</v>
+      </c>
+      <c r="J28" s="57">
+        <f>I28+J19</f>
+        <v/>
+      </c>
+      <c r="K28" s="57">
+        <f>J28+K19</f>
+        <v/>
+      </c>
+      <c r="L28" s="57">
+        <f>K28+L19</f>
+        <v/>
+      </c>
+      <c r="M28" s="57">
+        <f>L28+M19</f>
+        <v/>
+      </c>
+      <c r="N28" s="57">
+        <f>M28+N19</f>
+        <v/>
+      </c>
+      <c r="O28" s="57">
+        <f>N28+O19</f>
         <v/>
       </c>
       <c r="R28" s="44" t="inlineStr">
@@ -10656,34 +10650,55 @@
         <v/>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="40" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="J29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*1)/J24)</f>
-        <v/>
-      </c>
-      <c r="K29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*2)/K24)</f>
-        <v/>
-      </c>
-      <c r="L29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*3)/L24)</f>
-        <v/>
-      </c>
-      <c r="M29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*4)/M24)</f>
-        <v/>
-      </c>
-      <c r="N29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*5)/N24)</f>
-        <v/>
-      </c>
-      <c r="O29" s="59">
-        <f>MIN($C$6,($C$12+$C$9*6)/O24)</f>
+    <row r="29" hidden="1">
+      <c r="B29" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  occupied</t>
+        </is>
+      </c>
+      <c r="C29" s="57" t="n">
+        <v>11277</v>
+      </c>
+      <c r="D29" s="57" t="n">
+        <v>13152</v>
+      </c>
+      <c r="E29" s="57" t="n">
+        <v>14362</v>
+      </c>
+      <c r="F29" s="57" t="n">
+        <v>15047</v>
+      </c>
+      <c r="G29" s="57" t="n">
+        <v>17560</v>
+      </c>
+      <c r="H29" s="57" t="n">
+        <v>20215</v>
+      </c>
+      <c r="I29" s="57" t="n">
+        <v>22585</v>
+      </c>
+      <c r="J29" s="57">
+        <f>MIN($C$6*J28,I29+$C$11)</f>
+        <v/>
+      </c>
+      <c r="K29" s="57">
+        <f>MIN($C$6*K28,J29+$C$11)</f>
+        <v/>
+      </c>
+      <c r="L29" s="57">
+        <f>MIN($C$6*L28,K29+$C$11)</f>
+        <v/>
+      </c>
+      <c r="M29" s="57">
+        <f>MIN($C$6*M28,L29+$C$11)</f>
+        <v/>
+      </c>
+      <c r="N29" s="57">
+        <f>MIN($C$6*N28,M29+$C$11)</f>
+        <v/>
+      </c>
+      <c r="O29" s="57">
+        <f>MIN($C$6*O28,N29+$C$11)</f>
         <v/>
       </c>
       <c r="R29" s="44" t="inlineStr">
@@ -10714,35 +10729,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="40" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="J30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*1)/J24)</f>
-        <v/>
-      </c>
-      <c r="K30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*2)/K24)</f>
-        <v/>
-      </c>
-      <c r="L30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*3)/L24)</f>
-        <v/>
-      </c>
-      <c r="M30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*4)/M24)</f>
-        <v/>
-      </c>
-      <c r="N30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*5)/N24)</f>
-        <v/>
-      </c>
-      <c r="O30" s="59">
-        <f>MIN($C$6,($C$12+$C$10*6)/O24)</f>
-        <v/>
-      </c>
       <c r="R30" s="44" t="inlineStr">
         <is>
           <t>Sanctuair at Centerscape</t>
@@ -10771,6 +10757,41 @@
       </c>
     </row>
     <row r="31">
+      <c r="B31" s="40" t="inlineStr">
+        <is>
+          <t>IMPLIED 5-MI OCCUPANCY BY DEMAND SCENARIO</t>
+        </is>
+      </c>
+      <c r="J31" s="62" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="K31" s="62" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="L31" s="62" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="M31" s="62" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="N31" s="62" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="O31" s="62" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
       <c r="R31" s="44" t="inlineStr">
         <is>
           <t>Encore Avondale</t>
@@ -10805,38 +10826,32 @@
     <row r="32">
       <c r="B32" s="40" t="inlineStr">
         <is>
-          <t>MARKET RENT GROWTH (editable assumptions)</t>
-        </is>
-      </c>
-      <c r="J32" s="60" t="inlineStr">
-        <is>
-          <t>Y1</t>
-        </is>
-      </c>
-      <c r="K32" s="60" t="inlineStr">
-        <is>
-          <t>Y2</t>
-        </is>
-      </c>
-      <c r="L32" s="60" t="inlineStr">
-        <is>
-          <t>Y3</t>
-        </is>
-      </c>
-      <c r="M32" s="60" t="inlineStr">
-        <is>
-          <t>Y4</t>
-        </is>
-      </c>
-      <c r="N32" s="60" t="inlineStr">
-        <is>
-          <t>Y5</t>
-        </is>
-      </c>
-      <c r="O32" s="60" t="inlineStr">
-        <is>
-          <t>Y6</t>
-        </is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="J32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*1)/J28)</f>
+        <v/>
+      </c>
+      <c r="K32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*2)/K28)</f>
+        <v/>
+      </c>
+      <c r="L32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*3)/L28)</f>
+        <v/>
+      </c>
+      <c r="M32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*4)/M28)</f>
+        <v/>
+      </c>
+      <c r="N32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*5)/N28)</f>
+        <v/>
+      </c>
+      <c r="O32" s="63">
+        <f>MIN($C$6,($C$12+$C$8*6)/O28)</f>
+        <v/>
       </c>
       <c r="R32" s="44" t="inlineStr">
         <is>
@@ -10868,26 +10883,32 @@
     <row r="33">
       <c r="B33" s="40" t="inlineStr">
         <is>
-          <t>Bear</t>
-        </is>
-      </c>
-      <c r="J33" s="61" t="n">
-        <v>-0.0025</v>
-      </c>
-      <c r="K33" s="61" t="n">
-        <v>0.0175</v>
-      </c>
-      <c r="L33" s="61" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="M33" s="61" t="n">
-        <v>0.0375</v>
-      </c>
-      <c r="N33" s="61" t="n">
-        <v>0.0275</v>
-      </c>
-      <c r="O33" s="61" t="n">
-        <v>0.0175</v>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="J33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*1)/J28)</f>
+        <v/>
+      </c>
+      <c r="K33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*2)/K28)</f>
+        <v/>
+      </c>
+      <c r="L33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*3)/L28)</f>
+        <v/>
+      </c>
+      <c r="M33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*4)/M28)</f>
+        <v/>
+      </c>
+      <c r="N33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*5)/N28)</f>
+        <v/>
+      </c>
+      <c r="O33" s="63">
+        <f>MIN($C$6,($C$12+$C$9*6)/O28)</f>
+        <v/>
       </c>
       <c r="R33" s="44" t="inlineStr">
         <is>
@@ -10919,26 +10940,32 @@
     <row r="34">
       <c r="B34" s="40" t="inlineStr">
         <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="J34" s="61" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="K34" s="61" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="L34" s="61" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M34" s="61" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="N34" s="61" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="O34" s="61" t="n">
-        <v>0.03</v>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="J34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*1)/J28)</f>
+        <v/>
+      </c>
+      <c r="K34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*2)/K28)</f>
+        <v/>
+      </c>
+      <c r="L34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*3)/L28)</f>
+        <v/>
+      </c>
+      <c r="M34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*4)/M28)</f>
+        <v/>
+      </c>
+      <c r="N34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*5)/N28)</f>
+        <v/>
+      </c>
+      <c r="O34" s="63">
+        <f>MIN($C$6,($C$12+$C$10*6)/O28)</f>
+        <v/>
       </c>
       <c r="R34" s="44" t="inlineStr">
         <is>
@@ -10972,29 +10999,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="40" t="inlineStr">
-        <is>
-          <t>Bull</t>
-        </is>
-      </c>
-      <c r="J35" s="61" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="K35" s="61" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="L35" s="61" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="M35" s="61" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="N35" s="61" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="O35" s="61" t="n">
-        <v>0.04</v>
-      </c>
       <c r="R35" s="44" t="inlineStr">
         <is>
           <t>Orion Avondale</t>
@@ -11025,7 +11029,37 @@
     <row r="36">
       <c r="B36" s="40" t="inlineStr">
         <is>
-          <t>CONCESSIONS (months, editable)</t>
+          <t>MARKET RENT GROWTH (editable assumptions)</t>
+        </is>
+      </c>
+      <c r="J36" s="64" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="K36" s="64" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="L36" s="64" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="M36" s="64" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="N36" s="64" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="O36" s="64" t="inlineStr">
+        <is>
+          <t>Y6</t>
         </is>
       </c>
       <c r="R36" s="44" t="inlineStr">
@@ -11061,23 +11095,23 @@
           <t>Bear</t>
         </is>
       </c>
-      <c r="J37" s="61" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="K37" s="61" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="L37" s="61" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="M37" s="61" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="N37" s="61" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="O37" s="61" t="n">
-        <v>0.035</v>
+      <c r="J37" s="65" t="n">
+        <v>-0.0025</v>
+      </c>
+      <c r="K37" s="65" t="n">
+        <v>0.0175</v>
+      </c>
+      <c r="L37" s="65" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="M37" s="65" t="n">
+        <v>0.0375</v>
+      </c>
+      <c r="N37" s="65" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="O37" s="65" t="n">
+        <v>0.0175</v>
       </c>
       <c r="R37" s="44" t="inlineStr">
         <is>
@@ -11112,23 +11146,23 @@
           <t>Base</t>
         </is>
       </c>
-      <c r="J38" s="61" t="n">
+      <c r="J38" s="65" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K38" s="65" t="n">
         <v>0.03</v>
       </c>
-      <c r="K38" s="61" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="L38" s="61" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="M38" s="61" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="N38" s="61" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="O38" s="61" t="n">
-        <v>0.005</v>
+      <c r="L38" s="65" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M38" s="65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="N38" s="65" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="O38" s="65" t="n">
+        <v>0.03</v>
       </c>
       <c r="R38" s="44" t="inlineStr">
         <is>
@@ -11163,23 +11197,23 @@
           <t>Bull</t>
         </is>
       </c>
-      <c r="J39" s="61" t="n">
+      <c r="J39" s="65" t="n">
         <v>0.02</v>
       </c>
-      <c r="K39" s="61" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="L39" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="N39" s="61" t="n">
-        <v>0</v>
-      </c>
-      <c r="O39" s="61" t="n">
-        <v>0</v>
+      <c r="K39" s="65" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L39" s="65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M39" s="65" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="N39" s="65" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="O39" s="65" t="n">
+        <v>0.04</v>
       </c>
       <c r="R39" s="44" t="inlineStr">
         <is>
@@ -11211,7 +11245,7 @@
     <row r="40">
       <c r="B40" s="40" t="inlineStr">
         <is>
-          <t>EFFECTIVE RENT GROWTH (derived)</t>
+          <t>CONCESSIONS (months, editable)</t>
         </is>
       </c>
       <c r="R40" s="44" t="inlineStr">
@@ -11247,29 +11281,23 @@
           <t>Bear</t>
         </is>
       </c>
-      <c r="J41" s="59">
-        <f>(1+J33)*(1-J37)-1</f>
-        <v/>
-      </c>
-      <c r="K41" s="59">
-        <f>(1+K33)*(1-K37)/(1-J37)-1</f>
-        <v/>
-      </c>
-      <c r="L41" s="59">
-        <f>(1+L33)*(1-L37)/(1-K37)-1</f>
-        <v/>
-      </c>
-      <c r="M41" s="59">
-        <f>(1+M33)*(1-M37)/(1-L37)-1</f>
-        <v/>
-      </c>
-      <c r="N41" s="59">
-        <f>(1+N33)*(1-N37)/(1-M37)-1</f>
-        <v/>
-      </c>
-      <c r="O41" s="59">
-        <f>(1+O33)*(1-O37)/(1-N37)-1</f>
-        <v/>
+      <c r="J41" s="65" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K41" s="65" t="n">
+        <v>0.045</v>
+      </c>
+      <c r="L41" s="65" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="M41" s="65" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="N41" s="65" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="O41" s="65" t="n">
+        <v>0.035</v>
       </c>
       <c r="R41" s="44" t="inlineStr">
         <is>
@@ -11304,29 +11332,23 @@
           <t>Base</t>
         </is>
       </c>
-      <c r="J42" s="59">
-        <f>(1+J34)*(1-J38)-1</f>
-        <v/>
-      </c>
-      <c r="K42" s="59">
-        <f>(1+K34)*(1-K38)/(1-J38)-1</f>
-        <v/>
-      </c>
-      <c r="L42" s="59">
-        <f>(1+L34)*(1-L38)/(1-K38)-1</f>
-        <v/>
-      </c>
-      <c r="M42" s="59">
-        <f>(1+M34)*(1-M38)/(1-L38)-1</f>
-        <v/>
-      </c>
-      <c r="N42" s="59">
-        <f>(1+N34)*(1-N38)/(1-M38)-1</f>
-        <v/>
-      </c>
-      <c r="O42" s="59">
-        <f>(1+O34)*(1-O38)/(1-N38)-1</f>
-        <v/>
+      <c r="J42" s="65" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="K42" s="65" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="L42" s="65" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M42" s="65" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="N42" s="65" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="O42" s="65" t="n">
+        <v>0.005</v>
       </c>
       <c r="R42" s="44" t="inlineStr">
         <is>
@@ -11361,29 +11383,23 @@
           <t>Bull</t>
         </is>
       </c>
-      <c r="J43" s="59">
-        <f>(1+J35)*(1-J39)-1</f>
-        <v/>
-      </c>
-      <c r="K43" s="59">
-        <f>(1+K35)*(1-K39)/(1-J39)-1</f>
-        <v/>
-      </c>
-      <c r="L43" s="59">
-        <f>(1+L35)*(1-L39)/(1-K39)-1</f>
-        <v/>
-      </c>
-      <c r="M43" s="59">
-        <f>(1+M35)*(1-M39)/(1-L39)-1</f>
-        <v/>
-      </c>
-      <c r="N43" s="59">
-        <f>(1+N35)*(1-N39)/(1-M39)-1</f>
-        <v/>
-      </c>
-      <c r="O43" s="59">
-        <f>(1+O35)*(1-O39)/(1-N39)-1</f>
-        <v/>
+      <c r="J43" s="65" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K43" s="65" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L43" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="65" t="n">
+        <v>0</v>
+      </c>
+      <c r="O43" s="65" t="n">
+        <v>0</v>
       </c>
       <c r="R43" s="44" t="inlineStr">
         <is>
@@ -11413,9 +11429,9 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>Reconciliation: UC pipeline scheduled = 1,947 units vs CoStar current Under Construction = 1,251 units.</t>
+      <c r="B44" s="40" t="inlineStr">
+        <is>
+          <t>EFFECTIVE RENT GROWTH (derived)</t>
         </is>
       </c>
       <c r="R44" s="44" t="inlineStr">
@@ -11446,10 +11462,34 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="33" t="inlineStr">
-        <is>
-          <t>Note: as-of quarter (2026 Q2 QTD) is partial (quarter-to-date). Occupancy is point-in-time (valid); Y0 supply/absorption sums for that quarter are partial.</t>
-        </is>
+      <c r="B45" s="40" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="J45" s="63">
+        <f>(1+J37)*(1-J41)-1</f>
+        <v/>
+      </c>
+      <c r="K45" s="63">
+        <f>(1+K37)*(1-K41)/(1-J41)-1</f>
+        <v/>
+      </c>
+      <c r="L45" s="63">
+        <f>(1+L37)*(1-L41)/(1-K41)-1</f>
+        <v/>
+      </c>
+      <c r="M45" s="63">
+        <f>(1+M37)*(1-M41)/(1-L41)-1</f>
+        <v/>
+      </c>
+      <c r="N45" s="63">
+        <f>(1+N37)*(1-N41)/(1-M41)-1</f>
+        <v/>
+      </c>
+      <c r="O45" s="63">
+        <f>(1+O37)*(1-O41)/(1-N41)-1</f>
+        <v/>
       </c>
       <c r="R45" s="44" t="inlineStr">
         <is>
@@ -11479,10 +11519,34 @@
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="33" t="inlineStr">
-        <is>
-          <t>Historical = CoStar 5-mi TTM actuals. Forecast: inventory += UC (linked from Competitive Analysis) + proposed built this scenario; occupied += selected demand (capped at target). Yellow cells are editable.</t>
-        </is>
+      <c r="B46" s="40" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="J46" s="63">
+        <f>(1+J38)*(1-J42)-1</f>
+        <v/>
+      </c>
+      <c r="K46" s="63">
+        <f>(1+K38)*(1-K42)/(1-J42)-1</f>
+        <v/>
+      </c>
+      <c r="L46" s="63">
+        <f>(1+L38)*(1-L42)/(1-K42)-1</f>
+        <v/>
+      </c>
+      <c r="M46" s="63">
+        <f>(1+M38)*(1-M42)/(1-L42)-1</f>
+        <v/>
+      </c>
+      <c r="N46" s="63">
+        <f>(1+N38)*(1-N42)/(1-M42)-1</f>
+        <v/>
+      </c>
+      <c r="O46" s="63">
+        <f>(1+O38)*(1-O42)/(1-N42)-1</f>
+        <v/>
       </c>
       <c r="R46" s="44" t="inlineStr">
         <is>
@@ -11512,6 +11576,35 @@
       </c>
     </row>
     <row r="47">
+      <c r="B47" s="40" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="J47" s="63">
+        <f>(1+J39)*(1-J43)-1</f>
+        <v/>
+      </c>
+      <c r="K47" s="63">
+        <f>(1+K39)*(1-K43)/(1-J43)-1</f>
+        <v/>
+      </c>
+      <c r="L47" s="63">
+        <f>(1+L39)*(1-L43)/(1-K43)-1</f>
+        <v/>
+      </c>
+      <c r="M47" s="63">
+        <f>(1+M39)*(1-M43)/(1-L43)-1</f>
+        <v/>
+      </c>
+      <c r="N47" s="63">
+        <f>(1+N39)*(1-N43)/(1-M43)-1</f>
+        <v/>
+      </c>
+      <c r="O47" s="63">
+        <f>(1+O39)*(1-O43)/(1-N43)-1</f>
+        <v/>
+      </c>
       <c r="R47" s="44" t="inlineStr">
         <is>
           <t>Ascent Goodyear</t>
@@ -11544,6 +11637,11 @@
       </c>
     </row>
     <row r="48">
+      <c r="B48" s="33" t="inlineStr">
+        <is>
+          <t>Reconciliation: UC pipeline scheduled = 1,947 units vs CoStar current Under Construction = 1,251 units.</t>
+        </is>
+      </c>
       <c r="R48" s="44" t="inlineStr">
         <is>
           <t>Northern 107</t>
@@ -11576,6 +11674,11 @@
       </c>
     </row>
     <row r="49">
+      <c r="B49" s="33" t="inlineStr">
+        <is>
+          <t>Note: as-of quarter (2026 Q2 QTD) is partial (quarter-to-date). Occupancy is point-in-time (valid); Y0 supply/absorption sums for that quarter are partial.</t>
+        </is>
+      </c>
       <c r="R49" s="44" t="inlineStr">
         <is>
           <t>Zenn @ Sierra Verde</t>
@@ -11604,6 +11707,11 @@
       </c>
     </row>
     <row r="50">
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>Historical = CoStar 5-mi TTM actuals. Forecast: inventory += UC (linked from Competitive Analysis) + proposed built this scenario; occupied += selected demand (capped at target). Yellow cells are editable.</t>
+        </is>
+      </c>
       <c r="R50" s="44" t="inlineStr">
         <is>
           <t>The BLVD Residential District</t>

</xml_diff>

<commit_message>
Add Aura Beacon Island example; fix same-address mis-merge; fill occ gaps
- Reconciliation: guard against merging two distinct properties that share a
  street address (e.g. an existing asset and its planned redevelopment) — only
  merge when names share a real token, or year/units corroborate and there's no
  existing-vs-pipeline conflict. Fixes "Riverview at Clear Creek" (proposed) being
  fused with "Riverbend Apartment Homes" (1997 existing) at 301 N Wesley Dr.
- Subject rows: fill HelloData-window occupancy gaps from CoStar so the subject
  lease-up trajectory is continuous.
- Add examples/aura_beacon_island/ (League City, TX) and generated output.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Bella_Mirage__Supply_Chart.xlsx
+++ b/output/Bella_Mirage__Supply_Chart.xlsx
@@ -320,13 +320,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -738,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K118"/>
+  <dimension ref="B2:K120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="K16" s="8" t="inlineStr">
         <is>
-          <t>Year built: 2023/2024; Units: CoStar 292 vs RealPage 239; Delivery quarter estimated; Occ: CoStar 78% vs RealPage 87%</t>
+          <t>Year built: 2023/2024; Delivery quarter estimated; Occ: CoStar 78% vs RealPage 87%</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2673,7 @@
       </c>
       <c r="K53" s="15" t="inlineStr">
         <is>
-          <t>Delivery quarter estimated; Occ: CoStar 13% vs RealPage 0%; Rent: CoStar ask $1,411 vs RealPage eff $1,145; Verify rent/occ w/ HelloData</t>
+          <t>Delivery quarter estimated; Verify rent/occ w/ HelloData</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       <c r="B59" s="19" t="n"/>
       <c r="C59" s="20" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION (10 properties, 1,947 units)</t>
+          <t>UNDER CONSTRUCTION (11 properties, 2,307 units)</t>
         </is>
       </c>
     </row>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="C60" s="22" t="inlineStr">
         <is>
-          <t>FUZE Ballpark</t>
+          <t>Flatz623</t>
         </is>
       </c>
       <c r="D60" s="23" t="n">
-        <v>321</v>
+        <v>360</v>
       </c>
       <c r="E60" s="21" t="inlineStr">
         <is>
@@ -2876,7 +2876,7 @@
       <c r="I60" s="21" t="n"/>
       <c r="J60" s="21" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Low-Rise</t>
         </is>
       </c>
       <c r="K60" s="22" t="n"/>
@@ -2887,15 +2887,15 @@
       </c>
       <c r="C61" s="22" t="inlineStr">
         <is>
-          <t>HARMON Ascend</t>
+          <t>FUZE Ballpark</t>
         </is>
       </c>
       <c r="D61" s="23" t="n">
-        <v>125</v>
+        <v>321</v>
       </c>
       <c r="E61" s="21" t="inlineStr">
         <is>
-          <t>Q1 2027</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="F61" s="24" t="n"/>
@@ -2906,13 +2906,13 @@
       </c>
       <c r="H61" s="22" t="inlineStr">
         <is>
-          <t>Crescent Communities LLC</t>
+          <t>Zekelman Industries</t>
         </is>
       </c>
       <c r="I61" s="21" t="n"/>
       <c r="J61" s="21" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K61" s="22" t="n"/>
@@ -2923,15 +2923,15 @@
       </c>
       <c r="C62" s="22" t="inlineStr">
         <is>
-          <t>Pointe Grand Estrella at Phoenix</t>
+          <t>HARMON Ascend</t>
         </is>
       </c>
       <c r="D62" s="23" t="n">
-        <v>288</v>
+        <v>125</v>
       </c>
       <c r="E62" s="21" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q1 2027</t>
         </is>
       </c>
       <c r="F62" s="24" t="n"/>
@@ -2942,20 +2942,16 @@
       </c>
       <c r="H62" s="22" t="inlineStr">
         <is>
-          <t>Hillpointe, LLC</t>
+          <t>Crescent Communities LLC</t>
         </is>
       </c>
       <c r="I62" s="21" t="n"/>
       <c r="J62" s="21" t="inlineStr">
         <is>
-          <t>Garden</t>
-        </is>
-      </c>
-      <c r="K62" s="22" t="inlineStr">
-        <is>
-          <t>Year built: 2026/2027</t>
-        </is>
-      </c>
+          <t>Townhome</t>
+        </is>
+      </c>
+      <c r="K62" s="22" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="21" t="n">
@@ -2963,11 +2959,11 @@
       </c>
       <c r="C63" s="22" t="inlineStr">
         <is>
-          <t>Marbella Ranch East I</t>
+          <t>Pointe Grand Estrella at Phoenix</t>
         </is>
       </c>
       <c r="D63" s="23" t="n">
-        <v>144</v>
+        <v>288</v>
       </c>
       <c r="E63" s="21" t="inlineStr">
         <is>
@@ -2982,7 +2978,7 @@
       </c>
       <c r="H63" s="22" t="inlineStr">
         <is>
-          <t>Symmetry Companies</t>
+          <t>Hillpointe, LLC</t>
         </is>
       </c>
       <c r="I63" s="21" t="n"/>
@@ -2991,7 +2987,11 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K63" s="22" t="n"/>
+      <c r="K63" s="22" t="inlineStr">
+        <is>
+          <t>Year built: 2026/2027</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="B64" s="21" t="n">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="C64" s="22" t="inlineStr">
         <is>
-          <t>Villages at Northern</t>
+          <t>Marbella Ranch East I</t>
         </is>
       </c>
       <c r="D64" s="23" t="n">
-        <v>74</v>
+        <v>144</v>
       </c>
       <c r="E64" s="21" t="inlineStr">
         <is>
@@ -3018,7 +3018,7 @@
       </c>
       <c r="H64" s="22" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Symmetry Companies</t>
         </is>
       </c>
       <c r="I64" s="21" t="n"/>
@@ -3035,11 +3035,11 @@
       </c>
       <c r="C65" s="22" t="inlineStr">
         <is>
-          <t>Prosper 47</t>
+          <t>Villages at Northern</t>
         </is>
       </c>
       <c r="D65" s="23" t="n">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="E65" s="21" t="inlineStr">
         <is>
@@ -3060,14 +3060,10 @@
       <c r="I65" s="21" t="n"/>
       <c r="J65" s="21" t="inlineStr">
         <is>
-          <t>Townhome</t>
-        </is>
-      </c>
-      <c r="K65" s="22" t="inlineStr">
-        <is>
-          <t>RealPage only (sub-50 unit)</t>
-        </is>
-      </c>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K65" s="22" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="21" t="n">
@@ -3075,15 +3071,15 @@
       </c>
       <c r="C66" s="22" t="inlineStr">
         <is>
-          <t>Yardly Algodon</t>
+          <t>Prosper 47</t>
         </is>
       </c>
       <c r="D66" s="23" t="n">
-        <v>262</v>
+        <v>47</v>
       </c>
       <c r="E66" s="21" t="inlineStr">
         <is>
-          <t>Q4 2027</t>
+          <t>Q2 2027</t>
         </is>
       </c>
       <c r="F66" s="24" t="n"/>
@@ -3094,18 +3090,18 @@
       </c>
       <c r="H66" s="22" t="inlineStr">
         <is>
-          <t>Taylor Morrison, Inc.</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I66" s="21" t="n"/>
       <c r="J66" s="21" t="inlineStr">
         <is>
-          <t>Single Family</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K66" s="22" t="inlineStr">
         <is>
-          <t>Units: CoStar 262 vs RealPage 291; Year built: 2026/2027</t>
+          <t>RealPage only (sub-50 unit)</t>
         </is>
       </c>
     </row>
@@ -3115,11 +3111,11 @@
       </c>
       <c r="C67" s="22" t="inlineStr">
         <is>
-          <t>Cerro Vista</t>
+          <t>Yardly Algodon</t>
         </is>
       </c>
       <c r="D67" s="23" t="n">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="E67" s="21" t="inlineStr">
         <is>
@@ -3134,16 +3130,20 @@
       </c>
       <c r="H67" s="22" t="inlineStr">
         <is>
-          <t>Virtua Partners</t>
+          <t>Taylor Morrison, Inc.</t>
         </is>
       </c>
       <c r="I67" s="21" t="n"/>
       <c r="J67" s="21" t="inlineStr">
         <is>
-          <t>Low-Rise</t>
-        </is>
-      </c>
-      <c r="K67" s="22" t="n"/>
+          <t>Single Family</t>
+        </is>
+      </c>
+      <c r="K67" s="22" t="inlineStr">
+        <is>
+          <t>Units: CoStar 262 vs RealPage 291; Year built: 2026/2027</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="21" t="n">
@@ -3151,15 +3151,15 @@
       </c>
       <c r="C68" s="22" t="inlineStr">
         <is>
-          <t>Zanjero III</t>
+          <t>Cerro Vista</t>
         </is>
       </c>
       <c r="D68" s="23" t="n">
-        <v>301</v>
+        <v>255</v>
       </c>
       <c r="E68" s="21" t="inlineStr">
         <is>
-          <t>Q2 2028</t>
+          <t>Q4 2027</t>
         </is>
       </c>
       <c r="F68" s="24" t="n"/>
@@ -3170,13 +3170,13 @@
       </c>
       <c r="H68" s="22" t="inlineStr">
         <is>
-          <t>Fore Property Company/Privately Owned</t>
+          <t>Virtua Partners</t>
         </is>
       </c>
       <c r="I68" s="21" t="n"/>
       <c r="J68" s="21" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Low-Rise</t>
         </is>
       </c>
       <c r="K68" s="22" t="n"/>
@@ -3187,11 +3187,11 @@
       </c>
       <c r="C69" s="22" t="inlineStr">
         <is>
-          <t>Zen @ Angelina</t>
+          <t>Zanjero III</t>
         </is>
       </c>
       <c r="D69" s="23" t="n">
-        <v>130</v>
+        <v>301</v>
       </c>
       <c r="E69" s="21" t="inlineStr">
         <is>
@@ -3206,64 +3206,64 @@
       </c>
       <c r="H69" s="22" t="inlineStr">
         <is>
-          <t>F &amp; S Consulting &amp; Management, LLC</t>
+          <t>Fore Property Company/Privately Owned</t>
         </is>
       </c>
       <c r="I69" s="21" t="n"/>
       <c r="J69" s="21" t="inlineStr">
         <is>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
+      <c r="K69" s="22" t="n"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="21" t="n">
+        <v>61</v>
+      </c>
+      <c r="C70" s="22" t="inlineStr">
+        <is>
+          <t>Zen @ Angelina</t>
+        </is>
+      </c>
+      <c r="D70" s="23" t="n">
+        <v>130</v>
+      </c>
+      <c r="E70" s="21" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="F70" s="24" t="n"/>
+      <c r="G70" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H70" s="22" t="inlineStr">
+        <is>
+          <t>F &amp; S Consulting &amp; Management, LLC</t>
+        </is>
+      </c>
+      <c r="I70" s="21" t="n"/>
+      <c r="J70" s="21" t="inlineStr">
+        <is>
           <t>Townhome</t>
         </is>
       </c>
-      <c r="K69" s="22" t="inlineStr">
+      <c r="K70" s="22" t="inlineStr">
         <is>
           <t>Year built: 2027/2028</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="B71" s="26" t="n"/>
-      <c r="C71" s="27" t="inlineStr">
-        <is>
-          <t>PROPOSED (44 properties, 8,986 units)</t>
-        </is>
-      </c>
-    </row>
     <row r="72">
-      <c r="B72" s="28" t="n">
-        <v>61</v>
-      </c>
-      <c r="C72" s="29" t="inlineStr">
-        <is>
-          <t>The Waverly</t>
-        </is>
-      </c>
-      <c r="D72" s="30" t="n">
-        <v>323</v>
-      </c>
-      <c r="E72" s="28" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="F72" s="31" t="n"/>
-      <c r="G72" s="32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H72" s="29" t="inlineStr">
-        <is>
-          <t>Dominium</t>
-        </is>
-      </c>
-      <c r="I72" s="28" t="n"/>
-      <c r="J72" s="28" t="inlineStr">
-        <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
-      <c r="K72" s="29" t="n"/>
+      <c r="B72" s="26" t="n"/>
+      <c r="C72" s="27" t="inlineStr">
+        <is>
+          <t>PROPOSED (45 properties, 9,225 units)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="28" t="n">
@@ -3271,11 +3271,11 @@
       </c>
       <c r="C73" s="29" t="inlineStr">
         <is>
-          <t>Encore Avondale</t>
+          <t>The Waverly</t>
         </is>
       </c>
       <c r="D73" s="30" t="n">
-        <v>300</v>
+        <v>323</v>
       </c>
       <c r="E73" s="28" t="inlineStr">
         <is>
@@ -3290,7 +3290,7 @@
       </c>
       <c r="H73" s="29" t="inlineStr">
         <is>
-          <t>Encore Enterprises</t>
+          <t>Dominium</t>
         </is>
       </c>
       <c r="I73" s="28" t="n"/>
@@ -3307,11 +3307,11 @@
       </c>
       <c r="C74" s="29" t="inlineStr">
         <is>
-          <t>The Statler at Estrella Parkway</t>
+          <t>Encore Avondale</t>
         </is>
       </c>
       <c r="D74" s="30" t="n">
-        <v>284</v>
+        <v>300</v>
       </c>
       <c r="E74" s="28" t="inlineStr">
         <is>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="H74" s="29" t="inlineStr">
         <is>
-          <t>Leon Capital Group</t>
+          <t>Encore Enterprises</t>
         </is>
       </c>
       <c r="I74" s="28" t="n"/>
@@ -3343,11 +3343,11 @@
       </c>
       <c r="C75" s="29" t="inlineStr">
         <is>
-          <t>Ascent Goodyear</t>
+          <t>The Statler at Estrella Parkway</t>
         </is>
       </c>
       <c r="D75" s="30" t="n">
-        <v>113</v>
+        <v>284</v>
       </c>
       <c r="E75" s="28" t="inlineStr">
         <is>
@@ -3362,13 +3362,13 @@
       </c>
       <c r="H75" s="29" t="inlineStr">
         <is>
-          <t>Ascent Companies</t>
+          <t>Leon Capital Group</t>
         </is>
       </c>
       <c r="I75" s="28" t="n"/>
       <c r="J75" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K75" s="29" t="n"/>
@@ -3379,15 +3379,15 @@
       </c>
       <c r="C76" s="29" t="inlineStr">
         <is>
-          <t>Northern 107</t>
+          <t>Ascent Goodyear</t>
         </is>
       </c>
       <c r="D76" s="30" t="n">
-        <v>74</v>
+        <v>113</v>
       </c>
       <c r="E76" s="28" t="inlineStr">
         <is>
-          <t>Q4 2028</t>
+          <t>Q3 2028</t>
         </is>
       </c>
       <c r="F76" s="31" t="n"/>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="H76" s="29" t="inlineStr">
         <is>
-          <t>Jacob Reuben</t>
+          <t>Ascent Companies</t>
         </is>
       </c>
       <c r="I76" s="28" t="n"/>
@@ -3415,15 +3415,15 @@
       </c>
       <c r="C77" s="29" t="inlineStr">
         <is>
-          <t>Sheely Center Future Phase</t>
+          <t>Northern 107</t>
         </is>
       </c>
       <c r="D77" s="30" t="n">
-        <v>697</v>
+        <v>74</v>
       </c>
       <c r="E77" s="28" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q4 2028</t>
         </is>
       </c>
       <c r="F77" s="31" t="n"/>
@@ -3434,7 +3434,7 @@
       </c>
       <c r="H77" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Jacob Reuben</t>
         </is>
       </c>
       <c r="I77" s="28" t="n"/>
@@ -3443,11 +3443,7 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K77" s="29" t="inlineStr">
-        <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
-        </is>
-      </c>
+      <c r="K77" s="29" t="n"/>
     </row>
     <row r="78">
       <c r="B78" s="28" t="n">
@@ -3455,11 +3451,11 @@
       </c>
       <c r="C78" s="29" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel C</t>
+          <t>Sheely Center Future Phase</t>
         </is>
       </c>
       <c r="D78" s="30" t="n">
-        <v>500</v>
+        <v>697</v>
       </c>
       <c r="E78" s="28" t="inlineStr">
         <is>
@@ -3474,7 +3470,7 @@
       </c>
       <c r="H78" s="29" t="inlineStr">
         <is>
-          <t>Fisher Industries</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I78" s="28" t="n"/>
@@ -3495,11 +3491,11 @@
       </c>
       <c r="C79" s="29" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel B</t>
+          <t>Urban 95 Parcel C</t>
         </is>
       </c>
       <c r="D79" s="30" t="n">
-        <v>478</v>
+        <v>500</v>
       </c>
       <c r="E79" s="28" t="inlineStr">
         <is>
@@ -3520,7 +3516,7 @@
       <c r="I79" s="28" t="n"/>
       <c r="J79" s="28" t="inlineStr">
         <is>
-          <t>High-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K79" s="29" t="inlineStr">
@@ -3535,11 +3531,11 @@
       </c>
       <c r="C80" s="29" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel B</t>
+          <t>Urban 95 Parcel B</t>
         </is>
       </c>
       <c r="D80" s="30" t="n">
-        <v>410</v>
+        <v>478</v>
       </c>
       <c r="E80" s="28" t="inlineStr">
         <is>
@@ -3554,13 +3550,13 @@
       </c>
       <c r="H80" s="29" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>Fisher Industries</t>
         </is>
       </c>
       <c r="I80" s="28" t="n"/>
       <c r="J80" s="28" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>High-Rise</t>
         </is>
       </c>
       <c r="K80" s="29" t="inlineStr">
@@ -3575,11 +3571,11 @@
       </c>
       <c r="C81" s="29" t="inlineStr">
         <is>
-          <t>The District at Westgate</t>
+          <t>Celebration Plaza Parcel B</t>
         </is>
       </c>
       <c r="D81" s="30" t="n">
-        <v>384</v>
+        <v>410</v>
       </c>
       <c r="E81" s="28" t="inlineStr">
         <is>
@@ -3600,7 +3596,7 @@
       <c r="I81" s="28" t="n"/>
       <c r="J81" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K81" s="29" t="inlineStr">
@@ -3615,11 +3611,11 @@
       </c>
       <c r="C82" s="29" t="inlineStr">
         <is>
-          <t>Picerne at Palm Valley</t>
+          <t>The District at Westgate</t>
         </is>
       </c>
       <c r="D82" s="30" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E82" s="28" t="inlineStr">
         <is>
@@ -3634,7 +3630,7 @@
       </c>
       <c r="H82" s="29" t="inlineStr">
         <is>
-          <t>Picerne</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I82" s="28" t="n"/>
@@ -3655,11 +3651,11 @@
       </c>
       <c r="C83" s="29" t="inlineStr">
         <is>
-          <t>Liv Avondale</t>
+          <t>Picerne at Palm Valley</t>
         </is>
       </c>
       <c r="D83" s="30" t="n">
-        <v>333</v>
+        <v>383</v>
       </c>
       <c r="E83" s="28" t="inlineStr">
         <is>
@@ -3674,7 +3670,7 @@
       </c>
       <c r="H83" s="29" t="inlineStr">
         <is>
-          <t>Liv Communities LLC</t>
+          <t>Picerne</t>
         </is>
       </c>
       <c r="I83" s="28" t="n"/>
@@ -3695,11 +3691,11 @@
       </c>
       <c r="C84" s="29" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel A</t>
+          <t>Liv Avondale</t>
         </is>
       </c>
       <c r="D84" s="30" t="n">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="E84" s="28" t="inlineStr">
         <is>
@@ -3714,13 +3710,13 @@
       </c>
       <c r="H84" s="29" t="inlineStr">
         <is>
-          <t>Fisher Industries</t>
+          <t>Liv Communities LLC</t>
         </is>
       </c>
       <c r="I84" s="28" t="n"/>
       <c r="J84" s="28" t="inlineStr">
         <is>
-          <t>High-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K84" s="29" t="inlineStr">
@@ -3735,11 +3731,11 @@
       </c>
       <c r="C85" s="29" t="inlineStr">
         <is>
-          <t>Fuze 623</t>
+          <t>Urban 95 Parcel A</t>
         </is>
       </c>
       <c r="D85" s="30" t="n">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E85" s="28" t="inlineStr">
         <is>
@@ -3754,13 +3750,13 @@
       </c>
       <c r="H85" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Fisher Industries</t>
         </is>
       </c>
       <c r="I85" s="28" t="n"/>
       <c r="J85" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>High-Rise</t>
         </is>
       </c>
       <c r="K85" s="29" t="inlineStr">
@@ -3775,11 +3771,11 @@
       </c>
       <c r="C86" s="29" t="inlineStr">
         <is>
-          <t>Anton Glendale</t>
+          <t>Fuze 623</t>
         </is>
       </c>
       <c r="D86" s="30" t="n">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E86" s="28" t="inlineStr">
         <is>
@@ -3800,7 +3796,7 @@
       <c r="I86" s="28" t="n"/>
       <c r="J86" s="28" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K86" s="29" t="inlineStr">
@@ -3815,11 +3811,11 @@
       </c>
       <c r="C87" s="29" t="inlineStr">
         <is>
-          <t>Western Garden II</t>
+          <t>Anton Glendale</t>
         </is>
       </c>
       <c r="D87" s="30" t="n">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="E87" s="28" t="inlineStr">
         <is>
@@ -3834,13 +3830,13 @@
       </c>
       <c r="H87" s="29" t="inlineStr">
         <is>
-          <t>John F Long Properties LLLP</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I87" s="28" t="n"/>
       <c r="J87" s="28" t="inlineStr">
         <is>
-          <t>Single Family</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K87" s="29" t="inlineStr">
@@ -3855,11 +3851,11 @@
       </c>
       <c r="C88" s="29" t="inlineStr">
         <is>
-          <t>Sanctuair at Centerscape</t>
+          <t>Western Garden II</t>
         </is>
       </c>
       <c r="D88" s="30" t="n">
-        <v>303</v>
+        <v>314</v>
       </c>
       <c r="E88" s="28" t="inlineStr">
         <is>
@@ -3874,13 +3870,13 @@
       </c>
       <c r="H88" s="29" t="inlineStr">
         <is>
-          <t>Sunbelt Investment Holdings Inc</t>
+          <t>John F Long Properties LLLP</t>
         </is>
       </c>
       <c r="I88" s="28" t="n"/>
       <c r="J88" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Single Family</t>
         </is>
       </c>
       <c r="K88" s="29" t="inlineStr">
@@ -3895,11 +3891,11 @@
       </c>
       <c r="C89" s="29" t="inlineStr">
         <is>
-          <t>Banyan Avondale</t>
+          <t>Sanctuair at Centerscape</t>
         </is>
       </c>
       <c r="D89" s="30" t="n">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E89" s="28" t="inlineStr">
         <is>
@@ -3914,13 +3910,13 @@
       </c>
       <c r="H89" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sunbelt Investment Holdings Inc</t>
         </is>
       </c>
       <c r="I89" s="28" t="n"/>
       <c r="J89" s="28" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K89" s="29" t="inlineStr">
@@ -3935,11 +3931,11 @@
       </c>
       <c r="C90" s="29" t="inlineStr">
         <is>
-          <t>Rosilian Villas</t>
+          <t>Banyan Avondale</t>
         </is>
       </c>
       <c r="D90" s="30" t="n">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="E90" s="28" t="inlineStr">
         <is>
@@ -3960,7 +3956,7 @@
       <c r="I90" s="28" t="n"/>
       <c r="J90" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K90" s="29" t="inlineStr">
@@ -3975,11 +3971,11 @@
       </c>
       <c r="C91" s="29" t="inlineStr">
         <is>
-          <t>Orion Avondale</t>
+          <t>Rosilian Villas</t>
         </is>
       </c>
       <c r="D91" s="30" t="n">
-        <v>268</v>
+        <v>291</v>
       </c>
       <c r="E91" s="28" t="inlineStr">
         <is>
@@ -3994,13 +3990,13 @@
       </c>
       <c r="H91" s="29" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I91" s="28" t="n"/>
       <c r="J91" s="28" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K91" s="29" t="inlineStr">
@@ -4015,11 +4011,11 @@
       </c>
       <c r="C92" s="29" t="inlineStr">
         <is>
-          <t>Tavalo at Avondale</t>
+          <t>Orion Avondale</t>
         </is>
       </c>
       <c r="D92" s="30" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E92" s="28" t="inlineStr">
         <is>
@@ -4034,13 +4030,13 @@
       </c>
       <c r="H92" s="29" t="inlineStr">
         <is>
-          <t>GTIS Partners LP</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I92" s="28" t="n"/>
       <c r="J92" s="28" t="inlineStr">
         <is>
-          <t>Single Family</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K92" s="29" t="inlineStr">
@@ -4055,7 +4051,7 @@
       </c>
       <c r="C93" s="29" t="inlineStr">
         <is>
-          <t>Marbella Ranch East Future Phase</t>
+          <t>Tavalo at Avondale</t>
         </is>
       </c>
       <c r="D93" s="30" t="n">
@@ -4074,13 +4070,13 @@
       </c>
       <c r="H93" s="29" t="inlineStr">
         <is>
-          <t>Symmetry Companies</t>
+          <t>GTIS Partners LP</t>
         </is>
       </c>
       <c r="I93" s="28" t="n"/>
       <c r="J93" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Single Family</t>
         </is>
       </c>
       <c r="K93" s="29" t="inlineStr">
@@ -4095,11 +4091,11 @@
       </c>
       <c r="C94" s="29" t="inlineStr">
         <is>
-          <t>Crystal Cove</t>
+          <t>Marbella Ranch East Future Phase</t>
         </is>
       </c>
       <c r="D94" s="30" t="n">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="E94" s="28" t="inlineStr">
         <is>
@@ -4114,7 +4110,7 @@
       </c>
       <c r="H94" s="29" t="inlineStr">
         <is>
-          <t>Sterling Real Estate Partners</t>
+          <t>Symmetry Companies</t>
         </is>
       </c>
       <c r="I94" s="28" t="n"/>
@@ -4135,11 +4131,11 @@
       </c>
       <c r="C95" s="29" t="inlineStr">
         <is>
-          <t>Cornerstone at the Wigwam</t>
+          <t>Crystal Cove</t>
         </is>
       </c>
       <c r="D95" s="30" t="n">
-        <v>212</v>
+        <v>260</v>
       </c>
       <c r="E95" s="28" t="inlineStr">
         <is>
@@ -4154,13 +4150,13 @@
       </c>
       <c r="H95" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sterling Real Estate Partners</t>
         </is>
       </c>
       <c r="I95" s="28" t="n"/>
       <c r="J95" s="28" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K95" s="29" t="inlineStr">
@@ -4175,11 +4171,11 @@
       </c>
       <c r="C96" s="29" t="inlineStr">
         <is>
-          <t>Radia Avondale Station III</t>
+          <t>SimonMed Development I</t>
         </is>
       </c>
       <c r="D96" s="30" t="n">
-        <v>212</v>
+        <v>239</v>
       </c>
       <c r="E96" s="28" t="inlineStr">
         <is>
@@ -4215,11 +4211,11 @@
       </c>
       <c r="C97" s="29" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel A</t>
+          <t>Cornerstone at the Wigwam</t>
         </is>
       </c>
       <c r="D97" s="30" t="n">
-        <v>181</v>
+        <v>212</v>
       </c>
       <c r="E97" s="28" t="inlineStr">
         <is>
@@ -4234,7 +4230,7 @@
       </c>
       <c r="H97" s="29" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I97" s="28" t="n"/>
@@ -4255,11 +4251,11 @@
       </c>
       <c r="C98" s="29" t="inlineStr">
         <is>
-          <t>Villages at River Grove</t>
+          <t>Radia Avondale Station III</t>
         </is>
       </c>
       <c r="D98" s="30" t="n">
-        <v>180</v>
+        <v>212</v>
       </c>
       <c r="E98" s="28" t="inlineStr">
         <is>
@@ -4280,7 +4276,7 @@
       <c r="I98" s="28" t="n"/>
       <c r="J98" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K98" s="29" t="inlineStr">
@@ -4295,11 +4291,11 @@
       </c>
       <c r="C99" s="29" t="inlineStr">
         <is>
-          <t>District 99</t>
+          <t>Celebration Plaza Parcel A</t>
         </is>
       </c>
       <c r="D99" s="30" t="n">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="E99" s="28" t="inlineStr">
         <is>
@@ -4314,13 +4310,13 @@
       </c>
       <c r="H99" s="29" t="inlineStr">
         <is>
-          <t>Thompson Thrift</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I99" s="28" t="n"/>
       <c r="J99" s="28" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K99" s="29" t="inlineStr">
@@ -4335,11 +4331,11 @@
       </c>
       <c r="C100" s="29" t="inlineStr">
         <is>
-          <t>McDowell Villas</t>
+          <t>Villages at River Grove</t>
         </is>
       </c>
       <c r="D100" s="30" t="n">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="E100" s="28" t="inlineStr">
         <is>
@@ -4354,13 +4350,13 @@
       </c>
       <c r="H100" s="29" t="inlineStr">
         <is>
-          <t>Trilogy Investment Company</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I100" s="28" t="n"/>
       <c r="J100" s="28" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K100" s="29" t="inlineStr">
@@ -4375,11 +4371,11 @@
       </c>
       <c r="C101" s="29" t="inlineStr">
         <is>
-          <t>Avondale</t>
+          <t>District 99</t>
         </is>
       </c>
       <c r="D101" s="30" t="n">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="E101" s="28" t="inlineStr">
         <is>
@@ -4394,13 +4390,13 @@
       </c>
       <c r="H101" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Thompson Thrift</t>
         </is>
       </c>
       <c r="I101" s="28" t="n"/>
       <c r="J101" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K101" s="29" t="inlineStr">
@@ -4415,11 +4411,11 @@
       </c>
       <c r="C102" s="29" t="inlineStr">
         <is>
-          <t>Porter Kyle Development</t>
+          <t>McDowell Villas</t>
         </is>
       </c>
       <c r="D102" s="30" t="n">
-        <v>135</v>
+        <v>164</v>
       </c>
       <c r="E102" s="28" t="inlineStr">
         <is>
@@ -4434,7 +4430,7 @@
       </c>
       <c r="H102" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Trilogy Investment Company</t>
         </is>
       </c>
       <c r="I102" s="28" t="n"/>
@@ -4455,11 +4451,11 @@
       </c>
       <c r="C103" s="29" t="inlineStr">
         <is>
-          <t>Zenn @ Sierra Verde</t>
+          <t>Avondale</t>
         </is>
       </c>
       <c r="D103" s="30" t="n">
-        <v>66</v>
+        <v>156</v>
       </c>
       <c r="E103" s="28" t="inlineStr">
         <is>
@@ -4480,7 +4476,7 @@
       <c r="I103" s="28" t="n"/>
       <c r="J103" s="28" t="inlineStr">
         <is>
-          <t>Townhome</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K103" s="29" t="inlineStr">
@@ -4495,10 +4491,12 @@
       </c>
       <c r="C104" s="29" t="inlineStr">
         <is>
-          <t>The BLVD Residential District</t>
-        </is>
-      </c>
-      <c r="D104" s="30" t="n"/>
+          <t>Porter Kyle Development</t>
+        </is>
+      </c>
+      <c r="D104" s="30" t="n">
+        <v>135</v>
+      </c>
       <c r="E104" s="28" t="inlineStr">
         <is>
           <t>TBD</t>
@@ -4518,7 +4516,7 @@
       <c r="I104" s="28" t="n"/>
       <c r="J104" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K104" s="29" t="inlineStr">
@@ -4533,10 +4531,12 @@
       </c>
       <c r="C105" s="29" t="inlineStr">
         <is>
-          <t>The BLVD Park Avenue District</t>
-        </is>
-      </c>
-      <c r="D105" s="30" t="n"/>
+          <t>Zenn @ Sierra Verde</t>
+        </is>
+      </c>
+      <c r="D105" s="30" t="n">
+        <v>66</v>
+      </c>
       <c r="E105" s="28" t="inlineStr">
         <is>
           <t>TBD</t>
@@ -4556,7 +4556,7 @@
       <c r="I105" s="28" t="n"/>
       <c r="J105" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Townhome</t>
         </is>
       </c>
       <c r="K105" s="29" t="inlineStr">
@@ -4571,7 +4571,7 @@
       </c>
       <c r="C106" s="29" t="inlineStr">
         <is>
-          <t>Globe Land Investors Development</t>
+          <t>The BLVD Residential District</t>
         </is>
       </c>
       <c r="D106" s="30" t="n"/>
@@ -4588,7 +4588,7 @@
       </c>
       <c r="H106" s="29" t="inlineStr">
         <is>
-          <t>Globe Corporation</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I106" s="28" t="n"/>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="C107" s="29" t="inlineStr">
         <is>
-          <t>Ball Park</t>
+          <t>The BLVD Park Avenue District</t>
         </is>
       </c>
       <c r="D107" s="30" t="n"/>
@@ -4626,7 +4626,7 @@
       </c>
       <c r="H107" s="29" t="inlineStr">
         <is>
-          <t>VT LandGroup</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I107" s="28" t="n"/>
@@ -4647,7 +4647,7 @@
       </c>
       <c r="C108" s="29" t="inlineStr">
         <is>
-          <t>Vision 2 Parcel A</t>
+          <t>Globe Land Investors Development</t>
         </is>
       </c>
       <c r="D108" s="30" t="n"/>
@@ -4664,13 +4664,13 @@
       </c>
       <c r="H108" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Globe Corporation</t>
         </is>
       </c>
       <c r="I108" s="28" t="n"/>
       <c r="J108" s="28" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K108" s="29" t="inlineStr">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="C109" s="29" t="inlineStr">
         <is>
-          <t>Firststreet Verde</t>
+          <t>Ball Park</t>
         </is>
       </c>
       <c r="D109" s="30" t="n"/>
@@ -4702,13 +4702,13 @@
       </c>
       <c r="H109" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>VT LandGroup</t>
         </is>
       </c>
       <c r="I109" s="28" t="n"/>
       <c r="J109" s="28" t="inlineStr">
         <is>
-          <t>Single Family</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K109" s="29" t="inlineStr">
@@ -4723,7 +4723,7 @@
       </c>
       <c r="C110" s="29" t="inlineStr">
         <is>
-          <t>Goodyear Civic Square at Estrella Falls</t>
+          <t>Vision 2 Parcel A</t>
         </is>
       </c>
       <c r="D110" s="30" t="n"/>
@@ -4746,7 +4746,7 @@
       <c r="I110" s="28" t="n"/>
       <c r="J110" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Mid-Rise</t>
         </is>
       </c>
       <c r="K110" s="29" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="C111" s="29" t="inlineStr">
         <is>
-          <t>I-10 Innovation Center II</t>
+          <t>Firststreet Verde</t>
         </is>
       </c>
       <c r="D111" s="30" t="n"/>
@@ -4778,13 +4778,13 @@
       </c>
       <c r="H111" s="29" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I111" s="28" t="n"/>
       <c r="J111" s="28" t="inlineStr">
         <is>
-          <t>Garden</t>
+          <t>Single Family</t>
         </is>
       </c>
       <c r="K111" s="29" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="C112" s="29" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel D</t>
+          <t>Goodyear Civic Square at Estrella Falls</t>
         </is>
       </c>
       <c r="D112" s="30" t="n"/>
@@ -4816,7 +4816,7 @@
       </c>
       <c r="H112" s="29" t="inlineStr">
         <is>
-          <t>Privately Owned</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I112" s="28" t="n"/>
@@ -4837,7 +4837,7 @@
       </c>
       <c r="C113" s="29" t="inlineStr">
         <is>
-          <t>SimonMed Development II</t>
+          <t>I-10 Innovation Center II</t>
         </is>
       </c>
       <c r="D113" s="30" t="n"/>
@@ -4854,13 +4854,13 @@
       </c>
       <c r="H113" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I113" s="28" t="n"/>
       <c r="J113" s="28" t="inlineStr">
         <is>
-          <t>Mid-Rise</t>
+          <t>Garden</t>
         </is>
       </c>
       <c r="K113" s="29" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="C114" s="29" t="inlineStr">
         <is>
-          <t>182 South 95th Avenue</t>
+          <t>Celebration Plaza Parcel D</t>
         </is>
       </c>
       <c r="D114" s="30" t="n"/>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="H114" s="29" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Privately Owned</t>
         </is>
       </c>
       <c r="I114" s="28" t="n"/>
@@ -4913,7 +4913,7 @@
       </c>
       <c r="C115" s="29" t="inlineStr">
         <is>
-          <t>Envision Encore</t>
+          <t>SimonMed Development II</t>
         </is>
       </c>
       <c r="D115" s="30" t="n"/>
@@ -4936,17 +4936,93 @@
       <c r="I115" s="28" t="n"/>
       <c r="J115" s="28" t="inlineStr">
         <is>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
+      <c r="K115" s="29" t="inlineStr">
+        <is>
+          <t>RealPage pipeline (not yet in CoStar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="28" t="n">
+        <v>105</v>
+      </c>
+      <c r="C116" s="29" t="inlineStr">
+        <is>
+          <t>182 South 95th Avenue</t>
+        </is>
+      </c>
+      <c r="D116" s="30" t="n"/>
+      <c r="E116" s="28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F116" s="31" t="n"/>
+      <c r="G116" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H116" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I116" s="28" t="n"/>
+      <c r="J116" s="28" t="inlineStr">
+        <is>
           <t>Garden</t>
         </is>
       </c>
-      <c r="K115" s="29" t="inlineStr">
+      <c r="K116" s="29" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar)</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="B118" s="33" t="inlineStr">
+    <row r="117">
+      <c r="B117" s="28" t="n">
+        <v>106</v>
+      </c>
+      <c r="C117" s="29" t="inlineStr">
+        <is>
+          <t>Envision Encore</t>
+        </is>
+      </c>
+      <c r="D117" s="30" t="n"/>
+      <c r="E117" s="28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F117" s="31" t="n"/>
+      <c r="G117" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I117" s="28" t="n"/>
+      <c r="J117" s="28" t="inlineStr">
+        <is>
+          <t>Garden</t>
+        </is>
+      </c>
+      <c r="K117" s="29" t="inlineStr">
+        <is>
+          <t>RealPage pipeline (not yet in CoStar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="33" t="inlineStr">
         <is>
           <t>* 5-Mile radius. Rent ($) = market asking. Proximity (mi) to be filled manually; lease-up rent/occupancy to be verified w/ HelloData. See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
@@ -4955,11 +5031,11 @@
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="C59:K59"/>
-    <mergeCell ref="B118:K118"/>
+    <mergeCell ref="C72:K72"/>
     <mergeCell ref="C5:K5"/>
-    <mergeCell ref="C71:K71"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B120:K120"/>
     <mergeCell ref="C29:K29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4972,7 +5048,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z61"/>
+  <dimension ref="B1:Z63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -5096,15 +5172,15 @@
         <v>0.95</v>
       </c>
       <c r="R6" s="39">
-        <f>'Competitive Analysis'!C68</f>
+        <f>'Competitive Analysis'!C61</f>
         <v/>
       </c>
       <c r="S6" s="40">
-        <f>'Competitive Analysis'!D68</f>
+        <f>'Competitive Analysis'!D61</f>
         <v/>
       </c>
       <c r="T6" s="41">
-        <f>'Competitive Analysis'!E68</f>
+        <f>'Competitive Analysis'!E61</f>
         <v/>
       </c>
       <c r="V6">
@@ -5128,15 +5204,15 @@
         </is>
       </c>
       <c r="R7" s="39">
-        <f>'Competitive Analysis'!C62</f>
+        <f>'Competitive Analysis'!C69</f>
         <v/>
       </c>
       <c r="S7" s="40">
-        <f>'Competitive Analysis'!D62</f>
+        <f>'Competitive Analysis'!D69</f>
         <v/>
       </c>
       <c r="T7" s="41">
-        <f>'Competitive Analysis'!E62</f>
+        <f>'Competitive Analysis'!E69</f>
         <v/>
       </c>
       <c r="V7">
@@ -5158,15 +5234,15 @@
         <v>1250</v>
       </c>
       <c r="R8" s="39">
-        <f>'Competitive Analysis'!C66</f>
+        <f>'Competitive Analysis'!C63</f>
         <v/>
       </c>
       <c r="S8" s="40">
-        <f>'Competitive Analysis'!D66</f>
+        <f>'Competitive Analysis'!D63</f>
         <v/>
       </c>
       <c r="T8" s="41">
-        <f>'Competitive Analysis'!E66</f>
+        <f>'Competitive Analysis'!E63</f>
         <v/>
       </c>
       <c r="V8">
@@ -5218,15 +5294,15 @@
         <v>3800</v>
       </c>
       <c r="R10" s="39">
-        <f>'Competitive Analysis'!C63</f>
+        <f>'Competitive Analysis'!C68</f>
         <v/>
       </c>
       <c r="S10" s="40">
-        <f>'Competitive Analysis'!D63</f>
+        <f>'Competitive Analysis'!D68</f>
         <v/>
       </c>
       <c r="T10" s="41">
-        <f>'Competitive Analysis'!E63</f>
+        <f>'Competitive Analysis'!E68</f>
         <v/>
       </c>
       <c r="V10">
@@ -5249,15 +5325,15 @@
         <v/>
       </c>
       <c r="R11" s="39">
-        <f>'Competitive Analysis'!C69</f>
+        <f>'Competitive Analysis'!C64</f>
         <v/>
       </c>
       <c r="S11" s="40">
-        <f>'Competitive Analysis'!D69</f>
+        <f>'Competitive Analysis'!D64</f>
         <v/>
       </c>
       <c r="T11" s="41">
-        <f>'Competitive Analysis'!E69</f>
+        <f>'Competitive Analysis'!E64</f>
         <v/>
       </c>
       <c r="V11">
@@ -5271,15 +5347,15 @@
     </row>
     <row r="12" ht="14.4" customHeight="1">
       <c r="R12" s="39">
-        <f>'Competitive Analysis'!C61</f>
+        <f>'Competitive Analysis'!C70</f>
         <v/>
       </c>
       <c r="S12" s="40">
-        <f>'Competitive Analysis'!D61</f>
+        <f>'Competitive Analysis'!D70</f>
         <v/>
       </c>
       <c r="T12" s="41">
-        <f>'Competitive Analysis'!E61</f>
+        <f>'Competitive Analysis'!E70</f>
         <v/>
       </c>
       <c r="V12">
@@ -5293,15 +5369,15 @@
     </row>
     <row r="13" ht="14.4" customHeight="1">
       <c r="R13" s="39">
-        <f>'Competitive Analysis'!C64</f>
+        <f>'Competitive Analysis'!C62</f>
         <v/>
       </c>
       <c r="S13" s="40">
-        <f>'Competitive Analysis'!D64</f>
+        <f>'Competitive Analysis'!D62</f>
         <v/>
       </c>
       <c r="T13" s="41">
-        <f>'Competitive Analysis'!E64</f>
+        <f>'Competitive Analysis'!E62</f>
         <v/>
       </c>
       <c r="V13">
@@ -5335,14 +5411,29 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="14.4" customHeight="1"/>
-    <row r="16" ht="14.4" customHeight="1">
-      <c r="R16" s="34" t="inlineStr">
-        <is>
-          <t>PROPOSED PIPELINE (scenario toggle)</t>
-        </is>
-      </c>
-    </row>
+    <row r="15" ht="14.4" customHeight="1">
+      <c r="R15" s="39">
+        <f>'Competitive Analysis'!C66</f>
+        <v/>
+      </c>
+      <c r="S15" s="40">
+        <f>'Competitive Analysis'!D66</f>
+        <v/>
+      </c>
+      <c r="T15" s="41">
+        <f>'Competitive Analysis'!E66</f>
+        <v/>
+      </c>
+      <c r="V15">
+        <f>IFERROR(VALUE(RIGHT(T15,4))*4+MATCH(LEFT(T15,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W15">
+        <f>IF(V15="","",IF(V15&lt;=$Z$1,0,MAX(1,INT((V15-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="14.4" customHeight="1"/>
     <row r="17" ht="14.4" customHeight="1">
       <c r="B17" s="35" t="inlineStr">
         <is>
@@ -5414,24 +5505,9 @@
           <t>Y6</t>
         </is>
       </c>
-      <c r="R17" s="37" t="inlineStr">
-        <is>
-          <t>Property</t>
-        </is>
-      </c>
-      <c r="S17" s="37" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="T17" s="37" t="inlineStr">
-        <is>
-          <t>Est. Delivery</t>
-        </is>
-      </c>
-      <c r="U17" s="37" t="inlineStr">
-        <is>
-          <t>Built In</t>
+      <c r="R17" s="34" t="inlineStr">
+        <is>
+          <t>PROPOSED PIPELINE (scenario toggle)</t>
         </is>
       </c>
     </row>
@@ -5501,31 +5577,25 @@
           <t>Hold Yr 6</t>
         </is>
       </c>
-      <c r="R18" s="39" t="inlineStr">
-        <is>
-          <t>Sheely Center Future Phase</t>
-        </is>
-      </c>
-      <c r="S18" s="40" t="n">
-        <v>697</v>
-      </c>
-      <c r="T18" s="47" t="inlineStr"/>
-      <c r="U18" s="47" t="inlineStr">
-        <is>
-          <t>Bear only</t>
-        </is>
-      </c>
-      <c r="V18">
-        <f>IFERROR(VALUE(RIGHT(T18,4))*4+MATCH(LEFT(T18,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W18">
-        <f>IF(V18="","",IF(V18&lt;=$Z$1,0,MAX(1,INT((V18-$Z$2)/4)+1)))</f>
-        <v/>
-      </c>
-      <c r="X18">
-        <f>IF(U18="All",1,IF(U18="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U18="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
-        <v/>
+      <c r="R18" s="37" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="S18" s="37" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="T18" s="37" t="inlineStr">
+        <is>
+          <t>Est. Delivery</t>
+        </is>
+      </c>
+      <c r="U18" s="37" t="inlineStr">
+        <is>
+          <t>Built In</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="14.4" customHeight="1">
@@ -5534,61 +5604,61 @@
           <t>NEW SUPPLY (5-mi)</t>
         </is>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="47" t="n">
         <v>1133</v>
       </c>
-      <c r="D19" s="48" t="n">
+      <c r="D19" s="47" t="n">
         <v>1860</v>
       </c>
-      <c r="E19" s="48" t="n">
+      <c r="E19" s="47" t="n">
         <v>1336</v>
       </c>
-      <c r="F19" s="48" t="n">
+      <c r="F19" s="47" t="n">
         <v>2280</v>
       </c>
-      <c r="G19" s="48" t="n">
+      <c r="G19" s="47" t="n">
         <v>2823</v>
       </c>
-      <c r="H19" s="48" t="n">
+      <c r="H19" s="47" t="n">
         <v>4043</v>
       </c>
-      <c r="I19" s="48" t="n">
+      <c r="I19" s="47" t="n">
         <v>1860</v>
       </c>
-      <c r="J19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,1)+SUMIFS($S$18:$S$61,$W$18:$W$61,1,$X$18:$X$61,1)</f>
-        <v/>
-      </c>
-      <c r="K19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,2)+SUMIFS($S$18:$S$61,$W$18:$W$61,2,$X$18:$X$61,1)</f>
-        <v/>
-      </c>
-      <c r="L19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,3)+SUMIFS($S$18:$S$61,$W$18:$W$61,3,$X$18:$X$61,1)</f>
-        <v/>
-      </c>
-      <c r="M19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,4)+SUMIFS($S$18:$S$61,$W$18:$W$61,4,$X$18:$X$61,1)</f>
-        <v/>
-      </c>
-      <c r="N19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,5)+SUMIFS($S$18:$S$61,$W$18:$W$61,5,$X$18:$X$61,1)</f>
-        <v/>
-      </c>
-      <c r="O19" s="49">
-        <f>SUMIFS($S$5:$S$14,$W$5:$W$14,6)+SUMIFS($S$18:$S$61,$W$18:$W$61,6,$X$18:$X$61,1)</f>
+      <c r="J19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,1)+SUMIFS($S$19:$S$63,$W$19:$W$63,1,$X$19:$X$63,1)</f>
+        <v/>
+      </c>
+      <c r="K19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,2)+SUMIFS($S$19:$S$63,$W$19:$W$63,2,$X$19:$X$63,1)</f>
+        <v/>
+      </c>
+      <c r="L19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,3)+SUMIFS($S$19:$S$63,$W$19:$W$63,3,$X$19:$X$63,1)</f>
+        <v/>
+      </c>
+      <c r="M19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,4)+SUMIFS($S$19:$S$63,$W$19:$W$63,4,$X$19:$X$63,1)</f>
+        <v/>
+      </c>
+      <c r="N19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,5)+SUMIFS($S$19:$S$63,$W$19:$W$63,5,$X$19:$X$63,1)</f>
+        <v/>
+      </c>
+      <c r="O19" s="48">
+        <f>SUMIFS($S$5:$S$15,$W$5:$W$15,6)+SUMIFS($S$19:$S$63,$W$19:$W$63,6,$X$19:$X$63,1)</f>
         <v/>
       </c>
       <c r="R19" s="39" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel C</t>
+          <t>Sheely Center Future Phase</t>
         </is>
       </c>
       <c r="S19" s="40" t="n">
-        <v>500</v>
-      </c>
-      <c r="T19" s="47" t="inlineStr"/>
-      <c r="U19" s="47" t="inlineStr">
+        <v>697</v>
+      </c>
+      <c r="T19" s="49" t="inlineStr"/>
+      <c r="U19" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5612,61 +5682,61 @@
           <t>ABSORPTION (5-mi)</t>
         </is>
       </c>
-      <c r="C20" s="48" t="n">
+      <c r="C20" s="47" t="n">
         <v>719</v>
       </c>
-      <c r="D20" s="48" t="n">
+      <c r="D20" s="47" t="n">
         <v>1876</v>
       </c>
-      <c r="E20" s="48" t="n">
+      <c r="E20" s="47" t="n">
         <v>1210</v>
       </c>
-      <c r="F20" s="48" t="n">
+      <c r="F20" s="47" t="n">
         <v>685</v>
       </c>
-      <c r="G20" s="48" t="n">
+      <c r="G20" s="47" t="n">
         <v>2514</v>
       </c>
-      <c r="H20" s="48" t="n">
+      <c r="H20" s="47" t="n">
         <v>2655</v>
       </c>
-      <c r="I20" s="48" t="n">
+      <c r="I20" s="47" t="n">
         <v>2369</v>
       </c>
-      <c r="J20" s="49">
+      <c r="J20" s="48">
         <f>J31-I31</f>
         <v/>
       </c>
-      <c r="K20" s="49">
+      <c r="K20" s="48">
         <f>K31-J31</f>
         <v/>
       </c>
-      <c r="L20" s="49">
+      <c r="L20" s="48">
         <f>L31-K31</f>
         <v/>
       </c>
-      <c r="M20" s="49">
+      <c r="M20" s="48">
         <f>M31-L31</f>
         <v/>
       </c>
-      <c r="N20" s="49">
+      <c r="N20" s="48">
         <f>N31-M31</f>
         <v/>
       </c>
-      <c r="O20" s="49">
+      <c r="O20" s="48">
         <f>O31-N31</f>
         <v/>
       </c>
       <c r="R20" s="39" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel B</t>
+          <t>Urban 95 Parcel C</t>
         </is>
       </c>
       <c r="S20" s="40" t="n">
-        <v>478</v>
-      </c>
-      <c r="T20" s="47" t="inlineStr"/>
-      <c r="U20" s="47" t="inlineStr">
+        <v>500</v>
+      </c>
+      <c r="T20" s="49" t="inlineStr"/>
+      <c r="U20" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5737,14 +5807,14 @@
       </c>
       <c r="R21" s="39" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel B</t>
+          <t>Urban 95 Parcel B</t>
         </is>
       </c>
       <c r="S21" s="40" t="n">
-        <v>410</v>
-      </c>
-      <c r="T21" s="47" t="inlineStr"/>
-      <c r="U21" s="47" t="inlineStr">
+        <v>478</v>
+      </c>
+      <c r="T21" s="49" t="inlineStr"/>
+      <c r="U21" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5770,14 +5840,14 @@
       </c>
       <c r="R22" s="39" t="inlineStr">
         <is>
-          <t>The District at Westgate</t>
+          <t>Celebration Plaza Parcel B</t>
         </is>
       </c>
       <c r="S22" s="40" t="n">
-        <v>384</v>
-      </c>
-      <c r="T22" s="47" t="inlineStr"/>
-      <c r="U22" s="47" t="inlineStr">
+        <v>410</v>
+      </c>
+      <c r="T22" s="49" t="inlineStr"/>
+      <c r="U22" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5830,14 +5900,14 @@
       <c r="O23" s="53" t="n"/>
       <c r="R23" s="39" t="inlineStr">
         <is>
-          <t>Picerne at Palm Valley</t>
+          <t>The District at Westgate</t>
         </is>
       </c>
       <c r="S23" s="40" t="n">
-        <v>383</v>
-      </c>
-      <c r="T23" s="47" t="inlineStr"/>
-      <c r="U23" s="47" t="inlineStr">
+        <v>384</v>
+      </c>
+      <c r="T23" s="49" t="inlineStr"/>
+      <c r="U23" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5894,14 +5964,14 @@
       <c r="O24" s="56" t="n"/>
       <c r="R24" s="39" t="inlineStr">
         <is>
-          <t>Liv Avondale</t>
+          <t>Picerne at Palm Valley</t>
         </is>
       </c>
       <c r="S24" s="40" t="n">
-        <v>333</v>
-      </c>
-      <c r="T24" s="47" t="inlineStr"/>
-      <c r="U24" s="47" t="inlineStr">
+        <v>383</v>
+      </c>
+      <c r="T24" s="49" t="inlineStr"/>
+      <c r="U24" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -5954,14 +6024,14 @@
       <c r="O25" s="53" t="n"/>
       <c r="R25" s="39" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel A</t>
+          <t>Liv Avondale</t>
         </is>
       </c>
       <c r="S25" s="40" t="n">
-        <v>324</v>
-      </c>
-      <c r="T25" s="47" t="inlineStr"/>
-      <c r="U25" s="47" t="inlineStr">
+        <v>333</v>
+      </c>
+      <c r="T25" s="49" t="inlineStr"/>
+      <c r="U25" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6018,18 +6088,14 @@
       <c r="O26" s="56" t="n"/>
       <c r="R26" s="39" t="inlineStr">
         <is>
-          <t>The Waverly</t>
+          <t>Urban 95 Parcel A</t>
         </is>
       </c>
       <c r="S26" s="40" t="n">
-        <v>323</v>
-      </c>
-      <c r="T26" s="47" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U26" s="47" t="inlineStr">
+        <v>324</v>
+      </c>
+      <c r="T26" s="49" t="inlineStr"/>
+      <c r="U26" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6082,14 +6148,18 @@
       <c r="O27" s="58" t="n"/>
       <c r="R27" s="39" t="inlineStr">
         <is>
-          <t>Fuze 623</t>
+          <t>The Waverly</t>
         </is>
       </c>
       <c r="S27" s="40" t="n">
-        <v>321</v>
-      </c>
-      <c r="T27" s="47" t="inlineStr"/>
-      <c r="U27" s="47" t="inlineStr">
+        <v>323</v>
+      </c>
+      <c r="T27" s="49" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U27" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6140,14 +6210,14 @@
       <c r="O28" s="58" t="n"/>
       <c r="R28" s="39" t="inlineStr">
         <is>
-          <t>Anton Glendale</t>
+          <t>Fuze 623</t>
         </is>
       </c>
       <c r="S28" s="40" t="n">
-        <v>320</v>
-      </c>
-      <c r="T28" s="47" t="inlineStr"/>
-      <c r="U28" s="47" t="inlineStr">
+        <v>321</v>
+      </c>
+      <c r="T28" s="49" t="inlineStr"/>
+      <c r="U28" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6168,14 +6238,14 @@
     <row r="29" ht="14.4" customHeight="1">
       <c r="R29" s="39" t="inlineStr">
         <is>
-          <t>Western Garden II</t>
+          <t>Anton Glendale</t>
         </is>
       </c>
       <c r="S29" s="40" t="n">
-        <v>314</v>
-      </c>
-      <c r="T29" s="47" t="inlineStr"/>
-      <c r="U29" s="47" t="inlineStr">
+        <v>320</v>
+      </c>
+      <c r="T29" s="49" t="inlineStr"/>
+      <c r="U29" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6246,14 +6316,14 @@
       </c>
       <c r="R30" s="39" t="inlineStr">
         <is>
-          <t>Sanctuair at Centerscape</t>
+          <t>Western Garden II</t>
         </is>
       </c>
       <c r="S30" s="40" t="n">
-        <v>303</v>
-      </c>
-      <c r="T30" s="47" t="inlineStr"/>
-      <c r="U30" s="47" t="inlineStr">
+        <v>314</v>
+      </c>
+      <c r="T30" s="49" t="inlineStr"/>
+      <c r="U30" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6324,18 +6394,14 @@
       </c>
       <c r="R31" s="39" t="inlineStr">
         <is>
-          <t>Encore Avondale</t>
+          <t>Sanctuair at Centerscape</t>
         </is>
       </c>
       <c r="S31" s="40" t="n">
-        <v>300</v>
-      </c>
-      <c r="T31" s="47" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U31" s="47" t="inlineStr">
+        <v>303</v>
+      </c>
+      <c r="T31" s="49" t="inlineStr"/>
+      <c r="U31" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6356,14 +6422,18 @@
     <row r="32" ht="14.4" customHeight="1">
       <c r="R32" s="39" t="inlineStr">
         <is>
-          <t>Banyan Avondale</t>
+          <t>Encore Avondale</t>
         </is>
       </c>
       <c r="S32" s="40" t="n">
-        <v>296</v>
-      </c>
-      <c r="T32" s="47" t="inlineStr"/>
-      <c r="U32" s="47" t="inlineStr">
+        <v>300</v>
+      </c>
+      <c r="T32" s="49" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U32" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6419,14 +6489,14 @@
       </c>
       <c r="R33" s="39" t="inlineStr">
         <is>
-          <t>Rosilian Villas</t>
+          <t>Banyan Avondale</t>
         </is>
       </c>
       <c r="S33" s="40" t="n">
-        <v>291</v>
-      </c>
-      <c r="T33" s="47" t="inlineStr"/>
-      <c r="U33" s="47" t="inlineStr">
+        <v>296</v>
+      </c>
+      <c r="T33" s="49" t="inlineStr"/>
+      <c r="U33" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6476,18 +6546,14 @@
       </c>
       <c r="R34" s="39" t="inlineStr">
         <is>
-          <t>The Statler at Estrella Parkway</t>
+          <t>Rosilian Villas</t>
         </is>
       </c>
       <c r="S34" s="40" t="n">
-        <v>284</v>
-      </c>
-      <c r="T34" s="47" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U34" s="47" t="inlineStr">
+        <v>291</v>
+      </c>
+      <c r="T34" s="49" t="inlineStr"/>
+      <c r="U34" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6537,14 +6603,18 @@
       </c>
       <c r="R35" s="39" t="inlineStr">
         <is>
-          <t>Orion Avondale</t>
+          <t>The Statler at Estrella Parkway</t>
         </is>
       </c>
       <c r="S35" s="40" t="n">
-        <v>268</v>
-      </c>
-      <c r="T35" s="47" t="inlineStr"/>
-      <c r="U35" s="47" t="inlineStr">
+        <v>284</v>
+      </c>
+      <c r="T35" s="49" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U35" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6594,14 +6664,14 @@
       </c>
       <c r="R36" s="39" t="inlineStr">
         <is>
-          <t>Tavalo at Avondale</t>
+          <t>Orion Avondale</t>
         </is>
       </c>
       <c r="S36" s="40" t="n">
-        <v>266</v>
-      </c>
-      <c r="T36" s="47" t="inlineStr"/>
-      <c r="U36" s="47" t="inlineStr">
+        <v>268</v>
+      </c>
+      <c r="T36" s="49" t="inlineStr"/>
+      <c r="U36" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6622,14 +6692,14 @@
     <row r="37" ht="14.4" customHeight="1">
       <c r="R37" s="39" t="inlineStr">
         <is>
-          <t>Marbella Ranch East Future Phase</t>
+          <t>Tavalo at Avondale</t>
         </is>
       </c>
       <c r="S37" s="40" t="n">
         <v>266</v>
       </c>
-      <c r="T37" s="47" t="inlineStr"/>
-      <c r="U37" s="47" t="inlineStr">
+      <c r="T37" s="49" t="inlineStr"/>
+      <c r="U37" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6685,14 +6755,14 @@
       </c>
       <c r="R38" s="39" t="inlineStr">
         <is>
-          <t>Crystal Cove</t>
+          <t>Marbella Ranch East Future Phase</t>
         </is>
       </c>
       <c r="S38" s="40" t="n">
-        <v>260</v>
-      </c>
-      <c r="T38" s="47" t="inlineStr"/>
-      <c r="U38" s="47" t="inlineStr">
+        <v>266</v>
+      </c>
+      <c r="T38" s="49" t="inlineStr"/>
+      <c r="U38" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6736,14 +6806,14 @@
       </c>
       <c r="R39" s="39" t="inlineStr">
         <is>
-          <t>Cornerstone at the Wigwam</t>
+          <t>Crystal Cove</t>
         </is>
       </c>
       <c r="S39" s="40" t="n">
-        <v>212</v>
-      </c>
-      <c r="T39" s="47" t="inlineStr"/>
-      <c r="U39" s="47" t="inlineStr">
+        <v>260</v>
+      </c>
+      <c r="T39" s="49" t="inlineStr"/>
+      <c r="U39" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6787,14 +6857,14 @@
       </c>
       <c r="R40" s="39" t="inlineStr">
         <is>
-          <t>Radia Avondale Station III</t>
+          <t>SimonMed Development I</t>
         </is>
       </c>
       <c r="S40" s="40" t="n">
-        <v>212</v>
-      </c>
-      <c r="T40" s="47" t="inlineStr"/>
-      <c r="U40" s="47" t="inlineStr">
+        <v>239</v>
+      </c>
+      <c r="T40" s="49" t="inlineStr"/>
+      <c r="U40" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6838,14 +6908,14 @@
       </c>
       <c r="R41" s="39" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel A</t>
+          <t>Cornerstone at the Wigwam</t>
         </is>
       </c>
       <c r="S41" s="40" t="n">
-        <v>181</v>
-      </c>
-      <c r="T41" s="47" t="inlineStr"/>
-      <c r="U41" s="47" t="inlineStr">
+        <v>212</v>
+      </c>
+      <c r="T41" s="49" t="inlineStr"/>
+      <c r="U41" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6871,14 +6941,14 @@
       </c>
       <c r="R42" s="39" t="inlineStr">
         <is>
-          <t>Villages at River Grove</t>
+          <t>Radia Avondale Station III</t>
         </is>
       </c>
       <c r="S42" s="40" t="n">
-        <v>180</v>
-      </c>
-      <c r="T42" s="47" t="inlineStr"/>
-      <c r="U42" s="47" t="inlineStr">
+        <v>212</v>
+      </c>
+      <c r="T42" s="49" t="inlineStr"/>
+      <c r="U42" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6922,14 +6992,14 @@
       </c>
       <c r="R43" s="39" t="inlineStr">
         <is>
-          <t>District 99</t>
+          <t>Celebration Plaza Parcel A</t>
         </is>
       </c>
       <c r="S43" s="40" t="n">
-        <v>172</v>
-      </c>
-      <c r="T43" s="47" t="inlineStr"/>
-      <c r="U43" s="47" t="inlineStr">
+        <v>181</v>
+      </c>
+      <c r="T43" s="49" t="inlineStr"/>
+      <c r="U43" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -6973,14 +7043,14 @@
       </c>
       <c r="R44" s="39" t="inlineStr">
         <is>
-          <t>McDowell Villas</t>
+          <t>Villages at River Grove</t>
         </is>
       </c>
       <c r="S44" s="40" t="n">
-        <v>164</v>
-      </c>
-      <c r="T44" s="47" t="inlineStr"/>
-      <c r="U44" s="47" t="inlineStr">
+        <v>180</v>
+      </c>
+      <c r="T44" s="49" t="inlineStr"/>
+      <c r="U44" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7024,14 +7094,14 @@
       </c>
       <c r="R45" s="39" t="inlineStr">
         <is>
-          <t>Avondale</t>
+          <t>District 99</t>
         </is>
       </c>
       <c r="S45" s="40" t="n">
-        <v>156</v>
-      </c>
-      <c r="T45" s="47" t="inlineStr"/>
-      <c r="U45" s="47" t="inlineStr">
+        <v>172</v>
+      </c>
+      <c r="T45" s="49" t="inlineStr"/>
+      <c r="U45" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7057,14 +7127,14 @@
       </c>
       <c r="R46" s="39" t="inlineStr">
         <is>
-          <t>Porter Kyle Development</t>
+          <t>McDowell Villas</t>
         </is>
       </c>
       <c r="S46" s="40" t="n">
-        <v>135</v>
-      </c>
-      <c r="T46" s="47" t="inlineStr"/>
-      <c r="U46" s="47" t="inlineStr">
+        <v>164</v>
+      </c>
+      <c r="T46" s="49" t="inlineStr"/>
+      <c r="U46" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7114,18 +7184,14 @@
       </c>
       <c r="R47" s="39" t="inlineStr">
         <is>
-          <t>Ascent Goodyear</t>
+          <t>Avondale</t>
         </is>
       </c>
       <c r="S47" s="40" t="n">
-        <v>113</v>
-      </c>
-      <c r="T47" s="47" t="inlineStr">
-        <is>
-          <t>Q3 2028</t>
-        </is>
-      </c>
-      <c r="U47" s="47" t="inlineStr">
+        <v>156</v>
+      </c>
+      <c r="T47" s="49" t="inlineStr"/>
+      <c r="U47" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7175,18 +7241,14 @@
       </c>
       <c r="R48" s="39" t="inlineStr">
         <is>
-          <t>Northern 107</t>
+          <t>Porter Kyle Development</t>
         </is>
       </c>
       <c r="S48" s="40" t="n">
-        <v>74</v>
-      </c>
-      <c r="T48" s="47" t="inlineStr">
-        <is>
-          <t>Q4 2028</t>
-        </is>
-      </c>
-      <c r="U48" s="47" t="inlineStr">
+        <v>135</v>
+      </c>
+      <c r="T48" s="49" t="inlineStr"/>
+      <c r="U48" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7236,14 +7298,18 @@
       </c>
       <c r="R49" s="39" t="inlineStr">
         <is>
-          <t>Zenn @ Sierra Verde</t>
+          <t>Ascent Goodyear</t>
         </is>
       </c>
       <c r="S49" s="40" t="n">
-        <v>66</v>
-      </c>
-      <c r="T49" s="47" t="inlineStr"/>
-      <c r="U49" s="47" t="inlineStr">
+        <v>113</v>
+      </c>
+      <c r="T49" s="49" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
+      </c>
+      <c r="U49" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7264,12 +7330,18 @@
     <row r="50" ht="14.4" customHeight="1">
       <c r="R50" s="39" t="inlineStr">
         <is>
-          <t>The BLVD Residential District</t>
-        </is>
-      </c>
-      <c r="S50" s="40" t="n"/>
-      <c r="T50" s="47" t="inlineStr"/>
-      <c r="U50" s="47" t="inlineStr">
+          <t>Northern 107</t>
+        </is>
+      </c>
+      <c r="S50" s="40" t="n">
+        <v>74</v>
+      </c>
+      <c r="T50" s="49" t="inlineStr">
+        <is>
+          <t>Q4 2028</t>
+        </is>
+      </c>
+      <c r="U50" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7295,12 +7367,14 @@
       </c>
       <c r="R51" s="39" t="inlineStr">
         <is>
-          <t>The BLVD Park Avenue District</t>
-        </is>
-      </c>
-      <c r="S51" s="40" t="n"/>
-      <c r="T51" s="47" t="inlineStr"/>
-      <c r="U51" s="47" t="inlineStr">
+          <t>Zenn @ Sierra Verde</t>
+        </is>
+      </c>
+      <c r="S51" s="40" t="n">
+        <v>66</v>
+      </c>
+      <c r="T51" s="49" t="inlineStr"/>
+      <c r="U51" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7331,12 +7405,12 @@
       </c>
       <c r="R52" s="39" t="inlineStr">
         <is>
-          <t>Globe Land Investors Development</t>
+          <t>The BLVD Residential District</t>
         </is>
       </c>
       <c r="S52" s="40" t="n"/>
-      <c r="T52" s="47" t="inlineStr"/>
-      <c r="U52" s="47" t="inlineStr">
+      <c r="T52" s="49" t="inlineStr"/>
+      <c r="U52" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7367,12 +7441,12 @@
       </c>
       <c r="R53" s="39" t="inlineStr">
         <is>
-          <t>Ball Park</t>
+          <t>The BLVD Park Avenue District</t>
         </is>
       </c>
       <c r="S53" s="40" t="n"/>
-      <c r="T53" s="47" t="inlineStr"/>
-      <c r="U53" s="47" t="inlineStr">
+      <c r="T53" s="49" t="inlineStr"/>
+      <c r="U53" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7403,12 +7477,12 @@
       </c>
       <c r="R54" s="39" t="inlineStr">
         <is>
-          <t>Vision 2 Parcel A</t>
+          <t>Globe Land Investors Development</t>
         </is>
       </c>
       <c r="S54" s="40" t="n"/>
-      <c r="T54" s="47" t="inlineStr"/>
-      <c r="U54" s="47" t="inlineStr">
+      <c r="T54" s="49" t="inlineStr"/>
+      <c r="U54" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7439,12 +7513,12 @@
       </c>
       <c r="R55" s="39" t="inlineStr">
         <is>
-          <t>Firststreet Verde</t>
+          <t>Ball Park</t>
         </is>
       </c>
       <c r="S55" s="40" t="n"/>
-      <c r="T55" s="47" t="inlineStr"/>
-      <c r="U55" s="47" t="inlineStr">
+      <c r="T55" s="49" t="inlineStr"/>
+      <c r="U55" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7475,12 +7549,12 @@
       </c>
       <c r="R56" s="39" t="inlineStr">
         <is>
-          <t>Goodyear Civic Square at Estrella Falls</t>
+          <t>Vision 2 Parcel A</t>
         </is>
       </c>
       <c r="S56" s="40" t="n"/>
-      <c r="T56" s="47" t="inlineStr"/>
-      <c r="U56" s="47" t="inlineStr">
+      <c r="T56" s="49" t="inlineStr"/>
+      <c r="U56" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7511,12 +7585,12 @@
       </c>
       <c r="R57" s="39" t="inlineStr">
         <is>
-          <t>I-10 Innovation Center II</t>
+          <t>Firststreet Verde</t>
         </is>
       </c>
       <c r="S57" s="40" t="n"/>
-      <c r="T57" s="47" t="inlineStr"/>
-      <c r="U57" s="47" t="inlineStr">
+      <c r="T57" s="49" t="inlineStr"/>
+      <c r="U57" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7547,12 +7621,12 @@
       </c>
       <c r="R58" s="39" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel D</t>
+          <t>Goodyear Civic Square at Estrella Falls</t>
         </is>
       </c>
       <c r="S58" s="40" t="n"/>
-      <c r="T58" s="47" t="inlineStr"/>
-      <c r="U58" s="47" t="inlineStr">
+      <c r="T58" s="49" t="inlineStr"/>
+      <c r="U58" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7578,17 +7652,17 @@
       </c>
       <c r="E59" s="64" t="inlineStr">
         <is>
-          <t>1,947 / 1,251</t>
+          <t>2,307 / 1,251</t>
         </is>
       </c>
       <c r="R59" s="39" t="inlineStr">
         <is>
-          <t>SimonMed Development II</t>
+          <t>I-10 Innovation Center II</t>
         </is>
       </c>
       <c r="S59" s="40" t="n"/>
-      <c r="T59" s="47" t="inlineStr"/>
-      <c r="U59" s="47" t="inlineStr">
+      <c r="T59" s="49" t="inlineStr"/>
+      <c r="U59" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7614,12 +7688,12 @@
       </c>
       <c r="R60" s="39" t="inlineStr">
         <is>
-          <t>182 South 95th Avenue</t>
+          <t>Celebration Plaza Parcel D</t>
         </is>
       </c>
       <c r="S60" s="40" t="n"/>
-      <c r="T60" s="47" t="inlineStr"/>
-      <c r="U60" s="47" t="inlineStr">
+      <c r="T60" s="49" t="inlineStr"/>
+      <c r="U60" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7640,12 +7714,12 @@
     <row r="61" ht="14.4" customHeight="1">
       <c r="R61" s="39" t="inlineStr">
         <is>
-          <t>Envision Encore</t>
+          <t>SimonMed Development II</t>
         </is>
       </c>
       <c r="S61" s="40" t="n"/>
-      <c r="T61" s="47" t="inlineStr"/>
-      <c r="U61" s="47" t="inlineStr">
+      <c r="T61" s="49" t="inlineStr"/>
+      <c r="U61" s="49" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -7663,7 +7737,58 @@
         <v/>
       </c>
     </row>
-    <row r="62" ht="14.4" customHeight="1"/>
+    <row r="62" ht="14.4" customHeight="1">
+      <c r="R62" s="39" t="inlineStr">
+        <is>
+          <t>182 South 95th Avenue</t>
+        </is>
+      </c>
+      <c r="S62" s="40" t="n"/>
+      <c r="T62" s="49" t="inlineStr"/>
+      <c r="U62" s="49" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V62">
+        <f>IFERROR(VALUE(RIGHT(T62,4))*4+MATCH(LEFT(T62,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W62">
+        <f>IF(V62="","",IF(V62&lt;=$Z$1,0,MAX(1,INT((V62-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X62">
+        <f>IF(U62="All",1,IF(U62="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U62="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="R63" s="39" t="inlineStr">
+        <is>
+          <t>Envision Encore</t>
+        </is>
+      </c>
+      <c r="S63" s="40" t="n"/>
+      <c r="T63" s="49" t="inlineStr"/>
+      <c r="U63" s="49" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V63">
+        <f>IFERROR(VALUE(RIGHT(T63,4))*4+MATCH(LEFT(T63,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W63">
+        <f>IF(V63="","",IF(V63&lt;=$Z$1,0,MAX(1,INT((V63-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X63">
+        <f>IF(U63="All",1,IF(U63="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U63="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:O2"/>
@@ -7672,7 +7797,7 @@
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Bear,Base,Bull"</formula1>
     </dataValidation>
-    <dataValidation sqref="U18 U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U19 U20 U21 U22 U23 U24 U25 U26 U27 U28 U29 U30 U31 U32 U33 U34 U35 U36 U37 U38 U39 U40 U41 U42 U43 U44 U45 U46 U47 U48 U49 U50 U51 U52 U53 U54 U55 U56 U57 U58 U59 U60 U61 U62 U63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Bear only,Bear+Base,All,None"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7686,7 +7811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8157,7 +8282,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Year built: 2023/2024; Units: CoStar 292 vs RealPage 239; Delivery quarter estimated; Occ: CoStar 78% vs RealPage 87%</t>
+          <t>Year built: 2023/2024; Delivery quarter estimated; Occ: CoStar 78% vs RealPage 87%</t>
         </is>
       </c>
     </row>
@@ -9029,23 +9154,19 @@
       <c r="G27" s="66" t="n">
         <v>0.1333329999999999</v>
       </c>
-      <c r="H27" s="66" t="n">
-        <v>0</v>
-      </c>
+      <c r="H27" s="66" t="n"/>
       <c r="I27" s="67" t="n">
         <v>1411</v>
       </c>
-      <c r="J27" s="67" t="n">
-        <v>1145</v>
-      </c>
+      <c r="J27" s="67" t="n"/>
       <c r="K27" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
+          <t>CoStar</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Delivery quarter estimated; Occ: CoStar 13% vs RealPage 0%; Rent: CoStar ask $1,411 vs RealPage eff $1,145; Verify rent/occ w/ HelloData</t>
+          <t>Delivery quarter estimated; Verify rent/occ w/ HelloData</t>
         </is>
       </c>
     </row>
@@ -10638,34 +10759,41 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Northern 107</t>
+          <t>Flatz623</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>N 107th Ave</t>
+          <t>11850 W Fillmore St</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>74</v>
+        <v>360</v>
+      </c>
+      <c r="D62" t="n">
+        <v>2026</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Q4 2028</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
       <c r="G62" s="66" t="n"/>
-      <c r="H62" s="66" t="n"/>
+      <c r="H62" s="66" t="n">
+        <v>0</v>
+      </c>
       <c r="I62" s="67" t="n"/>
-      <c r="J62" s="67" t="n"/>
+      <c r="J62" s="67" t="n">
+        <v>1145</v>
+      </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>RealPage</t>
         </is>
       </c>
       <c r="L62" t="inlineStr"/>
@@ -10673,23 +10801,20 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>The Waverly</t>
+          <t>Northern 107</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>391 S 99th Ave</t>
+          <t>N 107th Ave</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>323</v>
-      </c>
-      <c r="D63" t="n">
-        <v>2028</v>
+        <v>74</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Q3 2028</t>
+          <t>Q4 2028</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -10703,7 +10828,7 @@
       <c r="J63" s="67" t="n"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
+          <t>CoStar</t>
         </is>
       </c>
       <c r="L63" t="inlineStr"/>
@@ -10711,16 +10836,19 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>The Statler at Estrella Parkway</t>
+          <t>The Waverly</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>240 N Estrella Pky</t>
+          <t>391 S 99th Ave</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>284</v>
+        <v>323</v>
+      </c>
+      <c r="D64" t="n">
+        <v>2028</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -10738,7 +10866,7 @@
       <c r="J64" s="67" t="n"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>CoStar+RealPage</t>
         </is>
       </c>
       <c r="L64" t="inlineStr"/>
@@ -10746,19 +10874,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Encore Avondale</t>
+          <t>The Statler at Estrella Parkway</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>11295 W Roosevelt St</t>
+          <t>240 N Estrella Pky</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>300</v>
-      </c>
-      <c r="D65" t="n">
-        <v>2027</v>
+        <v>284</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -10776,7 +10901,7 @@
       <c r="J65" s="67" t="n"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
+          <t>CoStar</t>
         </is>
       </c>
       <c r="L65" t="inlineStr"/>
@@ -10784,16 +10909,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Ascent Goodyear</t>
+          <t>Encore Avondale</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15681 W Roosevelt St</t>
+          <t>11295 W Roosevelt St</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>113</v>
+        <v>300</v>
       </c>
       <c r="D66" t="n">
         <v>2027</v>
@@ -10814,7 +10939,7 @@
       <c r="J66" s="67" t="n"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>CoStar+RealPage</t>
         </is>
       </c>
       <c r="L66" t="inlineStr"/>
@@ -10822,16 +10947,24 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>District 99</t>
+          <t>Ascent Goodyear</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>N 99th Ave &amp; W McDowell Rd</t>
+          <t>15681 W Roosevelt St</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>172</v>
+        <v>113</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2027</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Q3 2028</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -10844,28 +10977,24 @@
       <c r="J67" s="67" t="n"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>RealPage</t>
-        </is>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
-        </is>
-      </c>
+          <t>CoStar</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Liv Avondale</t>
+          <t>District 99</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>W Indian School Rd &amp; N 99th Ave</t>
+          <t>N 99th Ave &amp; W McDowell Rd</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>333</v>
+        <v>172</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -10890,16 +11019,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Sanctuair at Centerscape</t>
+          <t>Liv Avondale</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>1450 N 145th Ave</t>
+          <t>W Indian School Rd &amp; N 99th Ave</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>303</v>
+        <v>333</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -10924,16 +11053,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cornerstone at the Wigwam</t>
+          <t>Sanctuair at Centerscape</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Litchfield Rd &amp; Wigwam Blvd</t>
+          <t>1450 N 145th Ave</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>212</v>
+        <v>303</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -10958,13 +11087,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>The BLVD Residential District</t>
+          <t>Cornerstone at the Wigwam</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>W Roosevelt St &amp; W Hilton Way</t>
-        </is>
+          <t>Litchfield Rd &amp; Wigwam Blvd</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>212</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -10989,16 +11121,13 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Crystal Cove</t>
+          <t>The BLVD Residential District</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>290 E La Canada Blvd</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>260</v>
+          <t>W Roosevelt St &amp; W Hilton Way</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -11023,13 +11152,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>The BLVD Park Avenue District</t>
+          <t>Crystal Cove</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>N Avondale Blvd &amp; W Van Buren St</t>
-        </is>
+          <t>290 E La Canada Blvd</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>260</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -11054,16 +11186,13 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Western Garden II</t>
+          <t>The BLVD Park Avenue District</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>3301 N 99th Ave</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>314</v>
+          <t>N Avondale Blvd &amp; W Van Buren St</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -11088,16 +11217,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tavalo at Avondale</t>
+          <t>Western Garden II</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>12451 W Buckeye Rd</t>
+          <t>3301 N 99th Ave</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>266</v>
+        <v>314</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -11122,13 +11251,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Globe Land Investors Development</t>
+          <t>Tavalo at Avondale</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>N Bullard Ave &amp; W McDowell Rd</t>
-        </is>
+          <t>12451 W Buckeye Rd</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>266</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -11153,12 +11285,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Ball Park</t>
+          <t>Globe Land Investors Development</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>6450 N 99th Ave</t>
+          <t>N Bullard Ave &amp; W McDowell Rd</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -11184,16 +11316,13 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel B</t>
+          <t>Ball Park</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>N 95th Ave &amp; W Georgia Ave</t>
-        </is>
-      </c>
-      <c r="C78" t="n">
-        <v>478</v>
+          <t>6450 N 99th Ave</t>
+        </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -11218,16 +11347,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>The District at Westgate</t>
+          <t>Urban 95 Parcel B</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>6801 N 91st Ave</t>
+          <t>N 95th Ave &amp; W Georgia Ave</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>384</v>
+        <v>478</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -11252,13 +11381,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Vision 2 Parcel A</t>
+          <t>The District at Westgate</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>W Glendale Ave &amp; N 99th Ave</t>
-        </is>
+          <t>6801 N 91st Ave</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>384</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -11283,16 +11415,13 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Anton Glendale</t>
+          <t>Vision 2 Parcel A</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5149 &amp; 5205 N 99th Ave</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>320</v>
+          <t>W Glendale Ave &amp; N 99th Ave</t>
+        </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -11317,16 +11446,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Banyan Avondale</t>
+          <t>Anton Glendale</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Dysart Rd &amp; E Madison St</t>
+          <t>5149 &amp; 5205 N 99th Ave</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>296</v>
+        <v>320</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -11351,16 +11480,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel B</t>
+          <t>Banyan Avondale</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>844 Litchfield Rd</t>
+          <t>Dysart Rd &amp; E Madison St</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>410</v>
+        <v>296</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -11385,16 +11514,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel A</t>
+          <t>Celebration Plaza Parcel B</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>W Georgia Ave &amp; N 95th Ave</t>
+          <t>844 Litchfield Rd</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>324</v>
+        <v>410</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -11419,7 +11548,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Urban 95 Parcel C</t>
+          <t>Urban 95 Parcel A</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -11428,7 +11557,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>500</v>
+        <v>324</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -11453,13 +11582,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Firststreet Verde</t>
+          <t>Urban 95 Parcel C</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>9275 W Van Buren St</t>
-        </is>
+          <t>W Georgia Ave &amp; N 95th Ave</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>500</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -11484,16 +11616,13 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Radia Avondale Station III</t>
+          <t>Firststreet Verde</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>W Encanto Blvd &amp; N 99th Ave</t>
-        </is>
-      </c>
-      <c r="C87" t="n">
-        <v>212</v>
+          <t>9275 W Van Buren St</t>
+        </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -11518,16 +11647,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Rosilian Villas</t>
+          <t>Radia Avondale Station III</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>N Dysart Rd &amp; E Van Buren St</t>
+          <t>W Encanto Blvd &amp; N 99th Ave</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>291</v>
+        <v>212</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -11552,13 +11681,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Goodyear Civic Square at Estrella Falls</t>
+          <t>Rosilian Villas</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>W Monte Vista &amp; N 150th Dr</t>
-        </is>
+          <t>N Dysart Rd &amp; E Van Buren St</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>291</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -11583,12 +11715,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>I-10 Innovation Center II</t>
+          <t>Goodyear Civic Square at Estrella Falls</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>N 91st Ave &amp; W Roosevelt St</t>
+          <t>W Monte Vista &amp; N 150th Dr</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -11614,16 +11746,13 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Orion Avondale</t>
+          <t>I-10 Innovation Center II</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>W McDowell Rd &amp; Avondale Blvd</t>
-        </is>
-      </c>
-      <c r="C91" t="n">
-        <v>268</v>
+          <t>N 91st Ave &amp; W Roosevelt St</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -11648,16 +11777,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel A</t>
+          <t>Orion Avondale</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Celebrate Life Way &amp; N Litchfield Rd</t>
+          <t>W McDowell Rd &amp; Avondale Blvd</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>181</v>
+        <v>268</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -11682,13 +11811,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Celebration Plaza Parcel D</t>
+          <t>Celebration Plaza Parcel A</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
           <t>Celebrate Life Way &amp; N Litchfield Rd</t>
         </is>
+      </c>
+      <c r="C93" t="n">
+        <v>181</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -11713,16 +11845,13 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Sheely Center Future Phase</t>
+          <t>Celebration Plaza Parcel D</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2215 N 99th Ave</t>
-        </is>
-      </c>
-      <c r="C94" t="n">
-        <v>697</v>
+          <t>Celebrate Life Way &amp; N Litchfield Rd</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -11747,16 +11876,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Porter Kyle Development</t>
+          <t>Sheely Center Future Phase</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>W Camelback Rd &amp; S Denny Blvd</t>
+          <t>2215 N 99th Ave</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>135</v>
+        <v>697</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -11781,16 +11910,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>McDowell Villas</t>
+          <t>Porter Kyle Development</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>11791 W McDowell Rd</t>
+          <t>W Camelback Rd &amp; S Denny Blvd</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>164</v>
+        <v>135</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -11815,13 +11944,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SimonMed Development II</t>
+          <t>McDowell Villas</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>W Glendale Ave &amp; N 99th Ave</t>
-        </is>
+          <t>11791 W McDowell Rd</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>164</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -11846,12 +11978,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>182 South 95th Avenue</t>
+          <t>SimonMed Development II</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>182 S 95th Ave</t>
+          <t>W Glendale Ave &amp; N 99th Ave</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -11877,16 +12009,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Picerne at Palm Valley</t>
+          <t>SimonMed Development I</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2128 Pebble Creek Pkwy</t>
+          <t>10020 W Glendale Ave</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>383</v>
+        <v>239</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -11911,16 +12043,13 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Avondale</t>
+          <t>182 South 95th Avenue</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>1498 Historic US-80</t>
-        </is>
-      </c>
-      <c r="C100" t="n">
-        <v>156</v>
+          <t>182 S 95th Ave</t>
+        </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -11945,16 +12074,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Fuze 623</t>
+          <t>Picerne at Palm Valley</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>11745 W Corporate Dr</t>
+          <t>2128 Pebble Creek Pkwy</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>321</v>
+        <v>383</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -11979,16 +12108,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Villages at River Grove</t>
+          <t>Avondale</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>W Buckeye Rd &amp; S El Mirage Rd</t>
+          <t>1498 Historic US-80</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
@@ -12013,16 +12142,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Zenn @ Sierra Verde</t>
+          <t>Fuze 623</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>W Olive Ave &amp; N El Mirage Rd</t>
+          <t>11745 W Corporate Dr</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>66</v>
+        <v>321</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -12047,13 +12176,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Envision Encore</t>
+          <t>Villages at River Grove</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>N Ball Park Blvd &amp; N 99th Ave</t>
-        </is>
+          <t>W Buckeye Rd &amp; S El Mirage Rd</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>180</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -12078,16 +12210,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Marbella Ranch East Future Phase</t>
+          <t>Zenn @ Sierra Verde</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>W Northern Ave &amp; N El Mirage Rd</t>
+          <t>W Olive Ave &amp; N El Mirage Rd</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>266</v>
+        <v>66</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
@@ -12109,6 +12241,71 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Envision Encore</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>N Ball Park Blvd &amp; N 99th Ave</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="G106" s="66" t="n"/>
+      <c r="H106" s="66" t="n"/>
+      <c r="I106" s="67" t="n"/>
+      <c r="J106" s="67" t="n"/>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>RealPage</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>RealPage pipeline (not yet in CoStar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Marbella Ranch East Future Phase</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>W Northern Ave &amp; N El Mirage Rd</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>266</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="G107" s="66" t="n"/>
+      <c r="H107" s="66" t="n"/>
+      <c r="I107" s="67" t="n"/>
+      <c r="J107" s="67" t="n"/>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>RealPage</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>RealPage pipeline (not yet in CoStar)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>